<commit_message>
added r2 results data
</commit_message>
<xml_diff>
--- a/finalReport.xlsx
+++ b/finalReport.xlsx
@@ -5,18 +5,19 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fedev\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fedev\Documents\UNICAM\Phd\unmock\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FEFACB7-F48E-4046-83F1-38D15D89C311}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B5B9E6A-A321-4164-858C-8673DDB1DAD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{A0F7C0B4-A897-4B1D-9E87-712A814F4D93}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A0F7C0B4-A897-4B1D-9E87-712A814F4D93}"/>
   </bookViews>
   <sheets>
     <sheet name="r0" sheetId="1" r:id="rId1"/>
     <sheet name="r1" sheetId="2" r:id="rId2"/>
-    <sheet name="global" sheetId="4" r:id="rId3"/>
-    <sheet name="Test IDs" sheetId="3" r:id="rId4"/>
+    <sheet name="r2" sheetId="5" r:id="rId3"/>
+    <sheet name="global" sheetId="4" r:id="rId4"/>
+    <sheet name="Test IDs" sheetId="3" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="54">
   <si>
     <t>Target test</t>
   </si>
@@ -71,18 +72,6 @@
     <t>Transformed verify with semantic errors</t>
   </si>
   <si>
-    <t>Argument matchers in thenReturn</t>
-  </si>
-  <si>
-    <t>Transformed argument matchers in thenReturn</t>
-  </si>
-  <si>
-    <t>Transformed argument matchers in thenReturn with syntax errors</t>
-  </si>
-  <si>
-    <t>Transformed argument matcher in thenReturn with semantic errors</t>
-  </si>
-  <si>
     <t>Total mocked dependencies</t>
   </si>
   <si>
@@ -116,30 +105,6 @@
     <t>Cost ($)</t>
   </si>
   <si>
-    <t>0.023953</t>
-  </si>
-  <si>
-    <t>0.019517</t>
-  </si>
-  <si>
-    <t>0.011840</t>
-  </si>
-  <si>
-    <t>0.015064</t>
-  </si>
-  <si>
-    <t>0.012646</t>
-  </si>
-  <si>
-    <t>0.008600</t>
-  </si>
-  <si>
-    <t>0.011421</t>
-  </si>
-  <si>
-    <t>0.014811</t>
-  </si>
-  <si>
     <t>Needs human refactor (see Compilation errors for details)</t>
   </si>
   <si>
@@ -230,28 +195,16 @@
     <t>N.4</t>
   </si>
   <si>
-    <t>0.023829</t>
-  </si>
-  <si>
-    <t>0.024183</t>
-  </si>
-  <si>
-    <t>0.018274</t>
-  </si>
-  <si>
-    <t>0.018484</t>
-  </si>
-  <si>
-    <t>0.012227</t>
-  </si>
-  <si>
-    <t>0.009354</t>
-  </si>
-  <si>
-    <t>0.011980</t>
-  </si>
-  <si>
-    <t>0.014895</t>
+    <t>Argument matchers in stub</t>
+  </si>
+  <si>
+    <t>Transformed argument matchers in stub</t>
+  </si>
+  <si>
+    <t>Transformed argument matchers in stub with syntax errors</t>
+  </si>
+  <si>
+    <t>Transformed argument matcher in stub with semantic errors</t>
   </si>
 </sst>
 </file>
@@ -645,7 +598,7 @@
   <dimension ref="A1:I24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="61.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="55.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="9" width="11.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -920,7 +873,7 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>9</v>
+        <v>50</v>
       </c>
       <c r="B10">
         <v>0</v>
@@ -949,7 +902,7 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>10</v>
+        <v>51</v>
       </c>
       <c r="B11">
         <v>0</v>
@@ -978,7 +931,7 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>11</v>
+        <v>52</v>
       </c>
       <c r="B12">
         <v>0</v>
@@ -1007,7 +960,7 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>12</v>
+        <v>53</v>
       </c>
       <c r="B13">
         <v>0</v>
@@ -1036,7 +989,7 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B14">
         <v>3</v>
@@ -1065,7 +1018,7 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B15">
         <v>0</v>
@@ -1094,7 +1047,7 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B16">
         <v>3</v>
@@ -1123,7 +1076,7 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="B17">
         <v>3</v>
@@ -1152,7 +1105,7 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B18">
         <v>0</v>
@@ -1181,7 +1134,7 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B19">
         <v>0</v>
@@ -1210,7 +1163,7 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B20">
         <v>0</v>
@@ -1239,7 +1192,7 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B21" s="1">
         <v>22.84</v>
@@ -1268,89 +1221,89 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>21</v>
-      </c>
-      <c r="B22" t="s">
-        <v>22</v>
-      </c>
-      <c r="C22" t="s">
-        <v>22</v>
-      </c>
-      <c r="D22" t="s">
-        <v>22</v>
-      </c>
-      <c r="E22" t="s">
-        <v>22</v>
-      </c>
-      <c r="F22" t="s">
-        <v>22</v>
-      </c>
-      <c r="G22" t="s">
-        <v>22</v>
-      </c>
-      <c r="H22" t="s">
-        <v>22</v>
-      </c>
-      <c r="I22" t="s">
-        <v>22</v>
+        <v>19</v>
+      </c>
+      <c r="B22" s="1">
+        <v>2.3952999999999999E-2</v>
+      </c>
+      <c r="C22" s="1">
+        <v>2.3952999999999999E-2</v>
+      </c>
+      <c r="D22" s="1">
+        <v>2.3952999999999999E-2</v>
+      </c>
+      <c r="E22" s="1">
+        <v>2.3952999999999999E-2</v>
+      </c>
+      <c r="F22" s="1">
+        <v>2.3952999999999999E-2</v>
+      </c>
+      <c r="G22" s="1">
+        <v>2.3952999999999999E-2</v>
+      </c>
+      <c r="H22" s="1">
+        <v>2.3952999999999999E-2</v>
+      </c>
+      <c r="I22" s="1">
+        <v>2.3952999999999999E-2</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>23</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="G23" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="H23" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="I23" s="2" t="s">
-        <v>31</v>
+        <v>17</v>
+      </c>
+      <c r="B23" t="s">
+        <v>18</v>
+      </c>
+      <c r="C23" t="s">
+        <v>18</v>
+      </c>
+      <c r="D23" t="s">
+        <v>18</v>
+      </c>
+      <c r="E23" t="s">
+        <v>18</v>
+      </c>
+      <c r="F23" t="s">
+        <v>18</v>
+      </c>
+      <c r="G23" t="s">
+        <v>18</v>
+      </c>
+      <c r="H23" t="s">
+        <v>18</v>
+      </c>
+      <c r="I23" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="B24" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="C24" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="D24" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="E24" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="F24" t="s">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="G24" t="s">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="H24" t="s">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="I24" t="s">
-        <v>34</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -1363,7 +1316,7 @@
   <dimension ref="A1:I24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="61.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="55.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="9" width="11.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1638,7 +1591,7 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>9</v>
+        <v>50</v>
       </c>
       <c r="B10">
         <v>0</v>
@@ -1667,7 +1620,7 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>10</v>
+        <v>51</v>
       </c>
       <c r="B11">
         <v>0</v>
@@ -1696,7 +1649,7 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>11</v>
+        <v>52</v>
       </c>
       <c r="B12">
         <v>0</v>
@@ -1725,7 +1678,7 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>12</v>
+        <v>53</v>
       </c>
       <c r="B13">
         <v>0</v>
@@ -1754,7 +1707,7 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B14">
         <v>3</v>
@@ -1783,7 +1736,7 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B15">
         <v>0</v>
@@ -1812,7 +1765,7 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B16">
         <v>3</v>
@@ -1841,7 +1794,7 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="B17">
         <v>3</v>
@@ -1870,7 +1823,7 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B18">
         <v>0</v>
@@ -1899,7 +1852,7 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B19">
         <v>0</v>
@@ -1928,7 +1881,7 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B20">
         <v>0</v>
@@ -1957,7 +1910,7 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B21" s="1">
         <v>23.361999999999998</v>
@@ -1986,89 +1939,89 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>21</v>
-      </c>
-      <c r="B22" t="s">
-        <v>22</v>
-      </c>
-      <c r="C22" t="s">
-        <v>22</v>
-      </c>
-      <c r="D22" t="s">
-        <v>22</v>
-      </c>
-      <c r="E22" t="s">
-        <v>22</v>
-      </c>
-      <c r="F22" t="s">
-        <v>22</v>
-      </c>
-      <c r="G22" t="s">
-        <v>22</v>
-      </c>
-      <c r="H22" t="s">
-        <v>22</v>
-      </c>
-      <c r="I22" t="s">
-        <v>22</v>
+        <v>19</v>
+      </c>
+      <c r="B22" s="1">
+        <v>2.3828999999999999E-2</v>
+      </c>
+      <c r="C22" s="1">
+        <v>2.4183E-2</v>
+      </c>
+      <c r="D22" s="1">
+        <v>1.8273999999999999E-2</v>
+      </c>
+      <c r="E22" s="1">
+        <v>1.8484E-2</v>
+      </c>
+      <c r="F22" s="1">
+        <v>1.2227E-2</v>
+      </c>
+      <c r="G22" s="1">
+        <v>9.3539999999999995E-3</v>
+      </c>
+      <c r="H22" s="1">
+        <v>1.1979999999999999E-2</v>
+      </c>
+      <c r="I22" s="1">
+        <v>1.4895E-2</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>23</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="G23" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="H23" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="I23" s="2" t="s">
-        <v>69</v>
+        <v>17</v>
+      </c>
+      <c r="B23" t="s">
+        <v>18</v>
+      </c>
+      <c r="C23" t="s">
+        <v>18</v>
+      </c>
+      <c r="D23" t="s">
+        <v>18</v>
+      </c>
+      <c r="E23" t="s">
+        <v>18</v>
+      </c>
+      <c r="F23" t="s">
+        <v>18</v>
+      </c>
+      <c r="G23" t="s">
+        <v>18</v>
+      </c>
+      <c r="H23" t="s">
+        <v>18</v>
+      </c>
+      <c r="I23" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="B24" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="C24" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="D24" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="E24" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="F24" t="s">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="G24" t="s">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="H24" t="s">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="I24" t="s">
-        <v>34</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -2077,6 +2030,724 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B6A7EAB-DAE5-4AA9-9395-AE3C729544D4}">
+  <dimension ref="A1:I24"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="55.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="9" width="11.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="str">
+        <f>'Test IDs'!C2</f>
+        <v>DS.1</v>
+      </c>
+      <c r="C1" t="str">
+        <f>'Test IDs'!C3</f>
+        <v>DS.2</v>
+      </c>
+      <c r="D1" t="str">
+        <f>'Test IDs'!C4</f>
+        <v>DS.3</v>
+      </c>
+      <c r="E1" t="str">
+        <f>'Test IDs'!C5</f>
+        <v>DS.4</v>
+      </c>
+      <c r="F1" t="str">
+        <f>'Test IDs'!C6</f>
+        <v>N.1</v>
+      </c>
+      <c r="G1" t="str">
+        <f>'Test IDs'!C7</f>
+        <v>N.2</v>
+      </c>
+      <c r="H1" t="str">
+        <f>'Test IDs'!C8</f>
+        <v>N.3</v>
+      </c>
+      <c r="I1" t="str">
+        <f>'Test IDs'!C9</f>
+        <v>N.4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>3</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>3</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6">
+        <v>1</v>
+      </c>
+      <c r="I6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>0</v>
+      </c>
+      <c r="C7">
+        <v>2</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="G7">
+        <v>1</v>
+      </c>
+      <c r="H7">
+        <v>0</v>
+      </c>
+      <c r="I7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>0</v>
+      </c>
+      <c r="C8">
+        <v>0</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <v>0</v>
+      </c>
+      <c r="G8">
+        <v>1</v>
+      </c>
+      <c r="H8">
+        <v>1</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>0</v>
+      </c>
+      <c r="C9">
+        <v>0</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="F9">
+        <v>0</v>
+      </c>
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9">
+        <v>0</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>50</v>
+      </c>
+      <c r="B10">
+        <v>0</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <v>0</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <v>0</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>51</v>
+      </c>
+      <c r="B11">
+        <v>0</v>
+      </c>
+      <c r="C11">
+        <v>1</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11">
+        <v>0</v>
+      </c>
+      <c r="F11">
+        <v>0</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11">
+        <v>0</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>52</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12">
+        <v>0</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="F12">
+        <v>0</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="I12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>53</v>
+      </c>
+      <c r="B13">
+        <v>0</v>
+      </c>
+      <c r="C13">
+        <v>1</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+      <c r="F13">
+        <v>0</v>
+      </c>
+      <c r="G13">
+        <v>0</v>
+      </c>
+      <c r="H13">
+        <v>0</v>
+      </c>
+      <c r="I13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>9</v>
+      </c>
+      <c r="B14">
+        <v>3</v>
+      </c>
+      <c r="C14">
+        <v>1</v>
+      </c>
+      <c r="D14">
+        <v>1</v>
+      </c>
+      <c r="E14">
+        <v>1</v>
+      </c>
+      <c r="F14">
+        <v>1</v>
+      </c>
+      <c r="G14">
+        <v>1</v>
+      </c>
+      <c r="H14">
+        <v>1</v>
+      </c>
+      <c r="I14">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>10</v>
+      </c>
+      <c r="B15">
+        <v>0</v>
+      </c>
+      <c r="C15">
+        <v>0</v>
+      </c>
+      <c r="D15">
+        <v>0</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+      <c r="F15">
+        <v>1</v>
+      </c>
+      <c r="G15">
+        <v>0</v>
+      </c>
+      <c r="H15">
+        <v>1</v>
+      </c>
+      <c r="I15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>11</v>
+      </c>
+      <c r="B16">
+        <v>3</v>
+      </c>
+      <c r="C16">
+        <v>1</v>
+      </c>
+      <c r="D16">
+        <v>1</v>
+      </c>
+      <c r="E16">
+        <v>1</v>
+      </c>
+      <c r="F16">
+        <v>1</v>
+      </c>
+      <c r="G16">
+        <v>1</v>
+      </c>
+      <c r="H16">
+        <v>1</v>
+      </c>
+      <c r="I16">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>12</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17">
+        <v>1</v>
+      </c>
+      <c r="D17">
+        <v>1</v>
+      </c>
+      <c r="E17">
+        <v>1</v>
+      </c>
+      <c r="F17">
+        <v>1</v>
+      </c>
+      <c r="G17">
+        <v>1</v>
+      </c>
+      <c r="H17">
+        <v>1</v>
+      </c>
+      <c r="I17">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>13</v>
+      </c>
+      <c r="B18">
+        <v>3</v>
+      </c>
+      <c r="C18">
+        <v>2</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18">
+        <v>0</v>
+      </c>
+      <c r="F18">
+        <v>0</v>
+      </c>
+      <c r="G18">
+        <v>0</v>
+      </c>
+      <c r="H18">
+        <v>0</v>
+      </c>
+      <c r="I18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>14</v>
+      </c>
+      <c r="B19">
+        <v>0</v>
+      </c>
+      <c r="C19">
+        <v>0</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19">
+        <v>0</v>
+      </c>
+      <c r="F19">
+        <v>0</v>
+      </c>
+      <c r="G19">
+        <v>0</v>
+      </c>
+      <c r="H19">
+        <v>0</v>
+      </c>
+      <c r="I19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>15</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20">
+        <v>0</v>
+      </c>
+      <c r="D20">
+        <v>1</v>
+      </c>
+      <c r="E20">
+        <v>0</v>
+      </c>
+      <c r="F20">
+        <v>1</v>
+      </c>
+      <c r="G20">
+        <v>2</v>
+      </c>
+      <c r="H20">
+        <v>0</v>
+      </c>
+      <c r="I20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>16</v>
+      </c>
+      <c r="B21" s="1">
+        <v>30.553999999999998</v>
+      </c>
+      <c r="C21" s="1">
+        <v>20.238</v>
+      </c>
+      <c r="D21" s="1">
+        <v>13.242000000000001</v>
+      </c>
+      <c r="E21" s="1">
+        <v>16.619</v>
+      </c>
+      <c r="F21" s="1">
+        <v>12.702</v>
+      </c>
+      <c r="G21" s="1">
+        <v>9.4719999999999995</v>
+      </c>
+      <c r="H21" s="1">
+        <v>13.05</v>
+      </c>
+      <c r="I21" s="1">
+        <v>15.512</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>19</v>
+      </c>
+      <c r="B22" s="1">
+        <v>2.5378000000000001E-2</v>
+      </c>
+      <c r="C22" s="1">
+        <v>1.9817000000000001E-2</v>
+      </c>
+      <c r="D22" s="1">
+        <v>1.3224E-2</v>
+      </c>
+      <c r="E22" s="1">
+        <v>1.9071999999999999E-2</v>
+      </c>
+      <c r="F22" s="1">
+        <v>1.2208E-2</v>
+      </c>
+      <c r="G22" s="1">
+        <v>9.6340000000000002E-3</v>
+      </c>
+      <c r="H22" s="1">
+        <v>1.2047E-2</v>
+      </c>
+      <c r="I22" s="1">
+        <v>1.5117999999999999E-2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>17</v>
+      </c>
+      <c r="B23" t="s">
+        <v>18</v>
+      </c>
+      <c r="C23" t="s">
+        <v>18</v>
+      </c>
+      <c r="D23" t="s">
+        <v>18</v>
+      </c>
+      <c r="E23" t="s">
+        <v>18</v>
+      </c>
+      <c r="F23" t="s">
+        <v>18</v>
+      </c>
+      <c r="G23" t="s">
+        <v>18</v>
+      </c>
+      <c r="H23" t="s">
+        <v>18</v>
+      </c>
+      <c r="I23" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>20</v>
+      </c>
+      <c r="B24" t="s">
+        <v>22</v>
+      </c>
+      <c r="C24" t="s">
+        <v>22</v>
+      </c>
+      <c r="D24" t="s">
+        <v>22</v>
+      </c>
+      <c r="E24" t="s">
+        <v>21</v>
+      </c>
+      <c r="F24" t="s">
+        <v>22</v>
+      </c>
+      <c r="G24" t="s">
+        <v>22</v>
+      </c>
+      <c r="H24" t="s">
+        <v>22</v>
+      </c>
+      <c r="I24" t="s">
+        <v>22</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E040BF79-8B7D-43C4-816A-164CB83CAB3E}">
   <dimension ref="A1:I23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2127,35 +2798,35 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <f>AVERAGE(r0!B2,'r1'!B2)</f>
+        <f>AVERAGE(r0!B2,'r1'!B2, 'r2'!B2)</f>
         <v>3</v>
       </c>
       <c r="C2">
-        <f>AVERAGE(r0!C2,'r1'!C2)</f>
+        <f>AVERAGE(r0!C2,'r1'!C2, 'r2'!C2)</f>
         <v>2</v>
       </c>
       <c r="D2">
-        <f>AVERAGE(r0!D2,'r1'!D2)</f>
+        <f>AVERAGE(r0!D2,'r1'!D2, 'r2'!D2)</f>
         <v>1</v>
       </c>
       <c r="E2">
-        <f>AVERAGE(r0!E2,'r1'!E2)</f>
+        <f>AVERAGE(r0!E2,'r1'!E2, 'r2'!E2)</f>
         <v>1</v>
       </c>
       <c r="F2">
-        <f>AVERAGE(r0!F2,'r1'!F2)</f>
+        <f>AVERAGE(r0!F2,'r1'!F2, 'r2'!F2)</f>
         <v>1</v>
       </c>
       <c r="G2">
-        <f>AVERAGE(r0!G2,'r1'!G2)</f>
+        <f>AVERAGE(r0!G2,'r1'!G2, 'r2'!G2)</f>
         <v>0</v>
       </c>
       <c r="H2">
-        <f>AVERAGE(r0!H2,'r1'!H2)</f>
+        <f>AVERAGE(r0!H2,'r1'!H2, 'r2'!H2)</f>
         <v>0</v>
       </c>
       <c r="I2">
-        <f>AVERAGE(r0!I2,'r1'!I2)</f>
+        <f>AVERAGE(r0!I2,'r1'!I2, 'r2'!I2)</f>
         <v>1</v>
       </c>
     </row>
@@ -2164,35 +2835,35 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <f>AVERAGE(r0!B3,'r1'!B3)</f>
+        <f>AVERAGE(r0!B3,'r1'!B3, 'r2'!B3)</f>
         <v>3</v>
       </c>
       <c r="C3">
-        <f>AVERAGE(r0!C3,'r1'!C3)</f>
+        <f>AVERAGE(r0!C3,'r1'!C3, 'r2'!C3)</f>
         <v>2</v>
       </c>
       <c r="D3">
-        <f>AVERAGE(r0!D3,'r1'!D3)</f>
+        <f>AVERAGE(r0!D3,'r1'!D3, 'r2'!D3)</f>
         <v>1</v>
       </c>
       <c r="E3">
-        <f>AVERAGE(r0!E3,'r1'!E3)</f>
+        <f>AVERAGE(r0!E3,'r1'!E3, 'r2'!E3)</f>
         <v>1</v>
       </c>
       <c r="F3">
-        <f>AVERAGE(r0!F3,'r1'!F3)</f>
+        <f>AVERAGE(r0!F3,'r1'!F3, 'r2'!F3)</f>
         <v>1</v>
       </c>
       <c r="G3">
-        <f>AVERAGE(r0!G3,'r1'!G3)</f>
+        <f>AVERAGE(r0!G3,'r1'!G3, 'r2'!G3)</f>
         <v>0</v>
       </c>
       <c r="H3">
-        <f>AVERAGE(r0!H3,'r1'!H3)</f>
+        <f>AVERAGE(r0!H3,'r1'!H3, 'r2'!H3)</f>
         <v>0</v>
       </c>
       <c r="I3">
-        <f>AVERAGE(r0!I3,'r1'!I3)</f>
+        <f>AVERAGE(r0!I3,'r1'!I3, 'r2'!I3)</f>
         <v>1</v>
       </c>
     </row>
@@ -2201,35 +2872,35 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <f>AVERAGE(r0!B4,'r1'!B4)</f>
+        <f>AVERAGE(r0!B4,'r1'!B4, 'r2'!B4)</f>
         <v>0</v>
       </c>
       <c r="C4">
-        <f>AVERAGE(r0!C4,'r1'!C4)</f>
+        <f>AVERAGE(r0!C4,'r1'!C4, 'r2'!C4)</f>
         <v>0</v>
       </c>
       <c r="D4">
-        <f>AVERAGE(r0!D4,'r1'!D4)</f>
+        <f>AVERAGE(r0!D4,'r1'!D4, 'r2'!D4)</f>
         <v>0</v>
       </c>
       <c r="E4">
-        <f>AVERAGE(r0!E4,'r1'!E4)</f>
+        <f>AVERAGE(r0!E4,'r1'!E4, 'r2'!E4)</f>
         <v>0</v>
       </c>
       <c r="F4">
-        <f>AVERAGE(r0!F4,'r1'!F4)</f>
+        <f>AVERAGE(r0!F4,'r1'!F4, 'r2'!F4)</f>
         <v>0</v>
       </c>
       <c r="G4">
-        <f>AVERAGE(r0!G4,'r1'!G4)</f>
+        <f>AVERAGE(r0!G4,'r1'!G4, 'r2'!G4)</f>
         <v>0</v>
       </c>
       <c r="H4">
-        <f>AVERAGE(r0!H4,'r1'!H4)</f>
+        <f>AVERAGE(r0!H4,'r1'!H4, 'r2'!H4)</f>
         <v>0</v>
       </c>
       <c r="I4">
-        <f>AVERAGE(r0!I4,'r1'!I4)</f>
+        <f>AVERAGE(r0!I4,'r1'!I4, 'r2'!I4)</f>
         <v>0</v>
       </c>
     </row>
@@ -2238,35 +2909,35 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <f>AVERAGE(r0!B5,'r1'!B5)</f>
-        <v>0</v>
-      </c>
-      <c r="C5">
-        <f>AVERAGE(r0!C5,'r1'!C5)</f>
-        <v>0</v>
+        <f>AVERAGE(r0!B5,'r1'!B5, 'r2'!B5)</f>
+        <v>1</v>
+      </c>
+      <c r="C5" s="1">
+        <f>AVERAGE(r0!C5,'r1'!C5, 'r2'!C5)</f>
+        <v>0.33333333333333331</v>
       </c>
       <c r="D5">
-        <f>AVERAGE(r0!D5,'r1'!D5)</f>
+        <f>AVERAGE(r0!D5,'r1'!D5, 'r2'!D5)</f>
         <v>0</v>
       </c>
       <c r="E5">
-        <f>AVERAGE(r0!E5,'r1'!E5)</f>
+        <f>AVERAGE(r0!E5,'r1'!E5, 'r2'!E5)</f>
         <v>0</v>
       </c>
       <c r="F5">
-        <f>AVERAGE(r0!F5,'r1'!F5)</f>
+        <f>AVERAGE(r0!F5,'r1'!F5, 'r2'!F5)</f>
         <v>0</v>
       </c>
       <c r="G5">
-        <f>AVERAGE(r0!G5,'r1'!G5)</f>
+        <f>AVERAGE(r0!G5,'r1'!G5, 'r2'!G5)</f>
         <v>0</v>
       </c>
       <c r="H5">
-        <f>AVERAGE(r0!H5,'r1'!H5)</f>
+        <f>AVERAGE(r0!H5,'r1'!H5, 'r2'!H5)</f>
         <v>0</v>
       </c>
       <c r="I5">
-        <f>AVERAGE(r0!I5,'r1'!I5)</f>
+        <f>AVERAGE(r0!I5,'r1'!I5, 'r2'!I5)</f>
         <v>0</v>
       </c>
     </row>
@@ -2275,35 +2946,35 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <f>AVERAGE(r0!B6,'r1'!B6)</f>
+        <f>AVERAGE(r0!B6,'r1'!B6, 'r2'!B6)</f>
         <v>0</v>
       </c>
       <c r="C6">
-        <f>AVERAGE(r0!C6,'r1'!C6)</f>
+        <f>AVERAGE(r0!C6,'r1'!C6, 'r2'!C6)</f>
         <v>2</v>
       </c>
       <c r="D6">
-        <f>AVERAGE(r0!D6,'r1'!D6)</f>
+        <f>AVERAGE(r0!D6,'r1'!D6, 'r2'!D6)</f>
         <v>0</v>
       </c>
       <c r="E6">
-        <f>AVERAGE(r0!E6,'r1'!E6)</f>
+        <f>AVERAGE(r0!E6,'r1'!E6, 'r2'!E6)</f>
         <v>0</v>
       </c>
       <c r="F6">
-        <f>AVERAGE(r0!F6,'r1'!F6)</f>
+        <f>AVERAGE(r0!F6,'r1'!F6, 'r2'!F6)</f>
         <v>0</v>
       </c>
       <c r="G6">
-        <f>AVERAGE(r0!G6,'r1'!G6)</f>
+        <f>AVERAGE(r0!G6,'r1'!G6, 'r2'!G6)</f>
         <v>1</v>
       </c>
       <c r="H6">
-        <f>AVERAGE(r0!H6,'r1'!H6)</f>
+        <f>AVERAGE(r0!H6,'r1'!H6, 'r2'!H6)</f>
         <v>1</v>
       </c>
       <c r="I6">
-        <f>AVERAGE(r0!I6,'r1'!I6)</f>
+        <f>AVERAGE(r0!I6,'r1'!I6, 'r2'!I6)</f>
         <v>1</v>
       </c>
     </row>
@@ -2312,35 +2983,35 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <f>AVERAGE(r0!B7,'r1'!B7)</f>
+        <f>AVERAGE(r0!B7,'r1'!B7, 'r2'!B7)</f>
         <v>0</v>
       </c>
       <c r="C7">
-        <f>AVERAGE(r0!C7,'r1'!C7)</f>
+        <f>AVERAGE(r0!C7,'r1'!C7, 'r2'!C7)</f>
         <v>2</v>
       </c>
       <c r="D7">
-        <f>AVERAGE(r0!D7,'r1'!D7)</f>
+        <f>AVERAGE(r0!D7,'r1'!D7, 'r2'!D7)</f>
         <v>0</v>
       </c>
       <c r="E7">
-        <f>AVERAGE(r0!E7,'r1'!E7)</f>
+        <f>AVERAGE(r0!E7,'r1'!E7, 'r2'!E7)</f>
         <v>0</v>
       </c>
       <c r="F7">
-        <f>AVERAGE(r0!F7,'r1'!F7)</f>
+        <f>AVERAGE(r0!F7,'r1'!F7, 'r2'!F7)</f>
         <v>0</v>
       </c>
       <c r="G7">
-        <f>AVERAGE(r0!G7,'r1'!G7)</f>
-        <v>1</v>
-      </c>
-      <c r="H7">
-        <f>AVERAGE(r0!H7,'r1'!H7)</f>
-        <v>1</v>
+        <f>AVERAGE(r0!G7,'r1'!G7, 'r2'!G7)</f>
+        <v>1</v>
+      </c>
+      <c r="H7" s="1">
+        <f>AVERAGE(r0!H7,'r1'!H7, 'r2'!H7)</f>
+        <v>0.66666666666666663</v>
       </c>
       <c r="I7">
-        <f>AVERAGE(r0!I7,'r1'!I7)</f>
+        <f>AVERAGE(r0!I7,'r1'!I7, 'r2'!I7)</f>
         <v>1</v>
       </c>
     </row>
@@ -2349,35 +3020,35 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <f>AVERAGE(r0!B8,'r1'!B8)</f>
+        <f>AVERAGE(r0!B8,'r1'!B8, 'r2'!B8)</f>
         <v>0</v>
       </c>
       <c r="C8">
-        <f>AVERAGE(r0!C8,'r1'!C8)</f>
+        <f>AVERAGE(r0!C8,'r1'!C8, 'r2'!C8)</f>
         <v>0</v>
       </c>
       <c r="D8">
-        <f>AVERAGE(r0!D8,'r1'!D8)</f>
+        <f>AVERAGE(r0!D8,'r1'!D8, 'r2'!D8)</f>
         <v>0</v>
       </c>
       <c r="E8">
-        <f>AVERAGE(r0!E8,'r1'!E8)</f>
+        <f>AVERAGE(r0!E8,'r1'!E8, 'r2'!E8)</f>
         <v>0</v>
       </c>
       <c r="F8">
-        <f>AVERAGE(r0!F8,'r1'!F8)</f>
-        <v>0</v>
-      </c>
-      <c r="G8">
-        <f>AVERAGE(r0!G8,'r1'!G8)</f>
-        <v>0</v>
-      </c>
-      <c r="H8">
-        <f>AVERAGE(r0!H8,'r1'!H8)</f>
-        <v>0</v>
+        <f>AVERAGE(r0!F8,'r1'!F8, 'r2'!F8)</f>
+        <v>0</v>
+      </c>
+      <c r="G8" s="1">
+        <f>AVERAGE(r0!G8,'r1'!G8, 'r2'!G8)</f>
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="H8" s="1">
+        <f>AVERAGE(r0!H8,'r1'!H8, 'r2'!H8)</f>
+        <v>0.33333333333333331</v>
       </c>
       <c r="I8">
-        <f>AVERAGE(r0!I8,'r1'!I8)</f>
+        <f>AVERAGE(r0!I8,'r1'!I8, 'r2'!I8)</f>
         <v>0</v>
       </c>
     </row>
@@ -2386,480 +3057,517 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <f>AVERAGE(r0!B9,'r1'!B9)</f>
+        <f>AVERAGE(r0!B9,'r1'!B9, 'r2'!B9)</f>
         <v>0</v>
       </c>
       <c r="C9">
-        <f>AVERAGE(r0!C9,'r1'!C9)</f>
+        <f>AVERAGE(r0!C9,'r1'!C9, 'r2'!C9)</f>
         <v>0</v>
       </c>
       <c r="D9">
-        <f>AVERAGE(r0!D9,'r1'!D9)</f>
+        <f>AVERAGE(r0!D9,'r1'!D9, 'r2'!D9)</f>
         <v>0</v>
       </c>
       <c r="E9">
-        <f>AVERAGE(r0!E9,'r1'!E9)</f>
+        <f>AVERAGE(r0!E9,'r1'!E9, 'r2'!E9)</f>
         <v>0</v>
       </c>
       <c r="F9">
-        <f>AVERAGE(r0!F9,'r1'!F9)</f>
+        <f>AVERAGE(r0!F9,'r1'!F9, 'r2'!F9)</f>
         <v>0</v>
       </c>
       <c r="G9">
-        <f>AVERAGE(r0!G9,'r1'!G9)</f>
+        <f>AVERAGE(r0!G9,'r1'!G9, 'r2'!G9)</f>
         <v>0</v>
       </c>
       <c r="H9">
-        <f>AVERAGE(r0!H9,'r1'!H9)</f>
+        <f>AVERAGE(r0!H9,'r1'!H9, 'r2'!H9)</f>
         <v>0</v>
       </c>
       <c r="I9">
-        <f>AVERAGE(r0!I9,'r1'!I9)</f>
+        <f>AVERAGE(r0!I9,'r1'!I9, 'r2'!I9)</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>9</v>
+        <v>50</v>
       </c>
       <c r="B10">
-        <f>AVERAGE(r0!B10,'r1'!B10)</f>
+        <f>AVERAGE(r0!B10,'r1'!B10, 'r2'!B10)</f>
         <v>0</v>
       </c>
       <c r="C10">
-        <f>AVERAGE(r0!C10,'r1'!C10)</f>
+        <f>AVERAGE(r0!C10,'r1'!C10, 'r2'!C10)</f>
         <v>1</v>
       </c>
       <c r="D10">
-        <f>AVERAGE(r0!D10,'r1'!D10)</f>
+        <f>AVERAGE(r0!D10,'r1'!D10, 'r2'!D10)</f>
         <v>0</v>
       </c>
       <c r="E10">
-        <f>AVERAGE(r0!E10,'r1'!E10)</f>
+        <f>AVERAGE(r0!E10,'r1'!E10, 'r2'!E10)</f>
         <v>0</v>
       </c>
       <c r="F10">
-        <f>AVERAGE(r0!F10,'r1'!F10)</f>
+        <f>AVERAGE(r0!F10,'r1'!F10, 'r2'!F10)</f>
         <v>0</v>
       </c>
       <c r="G10">
-        <f>AVERAGE(r0!G10,'r1'!G10)</f>
+        <f>AVERAGE(r0!G10,'r1'!G10, 'r2'!G10)</f>
         <v>0</v>
       </c>
       <c r="H10">
-        <f>AVERAGE(r0!H10,'r1'!H10)</f>
+        <f>AVERAGE(r0!H10,'r1'!H10, 'r2'!H10)</f>
         <v>0</v>
       </c>
       <c r="I10">
-        <f>AVERAGE(r0!I10,'r1'!I10)</f>
+        <f>AVERAGE(r0!I10,'r1'!I10, 'r2'!I10)</f>
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>10</v>
+        <v>51</v>
       </c>
       <c r="B11">
-        <f>AVERAGE(r0!B11,'r1'!B11)</f>
-        <v>0</v>
-      </c>
-      <c r="C11">
-        <f>AVERAGE(r0!C11,'r1'!C11)</f>
-        <v>0.5</v>
+        <f>AVERAGE(r0!B11,'r1'!B11, 'r2'!B11)</f>
+        <v>0</v>
+      </c>
+      <c r="C11" s="1">
+        <f>AVERAGE(r0!C11,'r1'!C11, 'r2'!C11)</f>
+        <v>0.66666666666666663</v>
       </c>
       <c r="D11">
-        <f>AVERAGE(r0!D11,'r1'!D11)</f>
+        <f>AVERAGE(r0!D11,'r1'!D11, 'r2'!D11)</f>
         <v>0</v>
       </c>
       <c r="E11">
-        <f>AVERAGE(r0!E11,'r1'!E11)</f>
+        <f>AVERAGE(r0!E11,'r1'!E11, 'r2'!E11)</f>
         <v>0</v>
       </c>
       <c r="F11">
-        <f>AVERAGE(r0!F11,'r1'!F11)</f>
+        <f>AVERAGE(r0!F11,'r1'!F11, 'r2'!F11)</f>
         <v>0</v>
       </c>
       <c r="G11">
-        <f>AVERAGE(r0!G11,'r1'!G11)</f>
+        <f>AVERAGE(r0!G11,'r1'!G11, 'r2'!G11)</f>
         <v>0</v>
       </c>
       <c r="H11">
-        <f>AVERAGE(r0!H11,'r1'!H11)</f>
+        <f>AVERAGE(r0!H11,'r1'!H11, 'r2'!H11)</f>
         <v>0</v>
       </c>
       <c r="I11">
-        <f>AVERAGE(r0!I11,'r1'!I11)</f>
+        <f>AVERAGE(r0!I11,'r1'!I11, 'r2'!I11)</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>11</v>
+        <v>52</v>
       </c>
       <c r="B12">
-        <f>AVERAGE(r0!B12,'r1'!B12)</f>
+        <f>AVERAGE(r0!B12,'r1'!B12, 'r2'!B12)</f>
         <v>0</v>
       </c>
       <c r="C12">
-        <f>AVERAGE(r0!C12,'r1'!C12)</f>
+        <f>AVERAGE(r0!C12,'r1'!C12, 'r2'!C12)</f>
         <v>0</v>
       </c>
       <c r="D12">
-        <f>AVERAGE(r0!D12,'r1'!D12)</f>
+        <f>AVERAGE(r0!D12,'r1'!D12, 'r2'!D12)</f>
         <v>0</v>
       </c>
       <c r="E12">
-        <f>AVERAGE(r0!E12,'r1'!E12)</f>
+        <f>AVERAGE(r0!E12,'r1'!E12, 'r2'!E12)</f>
         <v>0</v>
       </c>
       <c r="F12">
-        <f>AVERAGE(r0!F12,'r1'!F12)</f>
+        <f>AVERAGE(r0!F12,'r1'!F12, 'r2'!F12)</f>
         <v>0</v>
       </c>
       <c r="G12">
-        <f>AVERAGE(r0!G12,'r1'!G12)</f>
+        <f>AVERAGE(r0!G12,'r1'!G12, 'r2'!G12)</f>
         <v>0</v>
       </c>
       <c r="H12">
-        <f>AVERAGE(r0!H12,'r1'!H12)</f>
+        <f>AVERAGE(r0!H12,'r1'!H12, 'r2'!H12)</f>
         <v>0</v>
       </c>
       <c r="I12">
-        <f>AVERAGE(r0!I12,'r1'!I12)</f>
+        <f>AVERAGE(r0!I12,'r1'!I12, 'r2'!I12)</f>
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>12</v>
+        <v>53</v>
       </c>
       <c r="B13">
-        <f>AVERAGE(r0!B13,'r1'!B13)</f>
-        <v>0</v>
-      </c>
-      <c r="C13">
-        <f>AVERAGE(r0!C13,'r1'!C13)</f>
-        <v>0</v>
+        <f>AVERAGE(r0!B13,'r1'!B13, 'r2'!B13)</f>
+        <v>0</v>
+      </c>
+      <c r="C13" s="1">
+        <f>AVERAGE(r0!C13,'r1'!C13, 'r2'!C13)</f>
+        <v>0.33333333333333331</v>
       </c>
       <c r="D13">
-        <f>AVERAGE(r0!D13,'r1'!D13)</f>
+        <f>AVERAGE(r0!D13,'r1'!D13, 'r2'!D13)</f>
         <v>0</v>
       </c>
       <c r="E13">
-        <f>AVERAGE(r0!E13,'r1'!E13)</f>
+        <f>AVERAGE(r0!E13,'r1'!E13, 'r2'!E13)</f>
         <v>0</v>
       </c>
       <c r="F13">
-        <f>AVERAGE(r0!F13,'r1'!F13)</f>
+        <f>AVERAGE(r0!F13,'r1'!F13, 'r2'!F13)</f>
         <v>0</v>
       </c>
       <c r="G13">
-        <f>AVERAGE(r0!G13,'r1'!G13)</f>
+        <f>AVERAGE(r0!G13,'r1'!G13, 'r2'!G13)</f>
         <v>0</v>
       </c>
       <c r="H13">
-        <f>AVERAGE(r0!H13,'r1'!H13)</f>
+        <f>AVERAGE(r0!H13,'r1'!H13, 'r2'!H13)</f>
         <v>0</v>
       </c>
       <c r="I13">
-        <f>AVERAGE(r0!I13,'r1'!I13)</f>
+        <f>AVERAGE(r0!I13,'r1'!I13, 'r2'!I13)</f>
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B14">
-        <f>AVERAGE(r0!B14,'r1'!B14)</f>
+        <f>AVERAGE(r0!B14,'r1'!B14, 'r2'!B14)</f>
         <v>3</v>
       </c>
       <c r="C14">
-        <f>AVERAGE(r0!C14,'r1'!C14)</f>
+        <f>AVERAGE(r0!C14,'r1'!C14, 'r2'!C14)</f>
         <v>1</v>
       </c>
       <c r="D14">
-        <f>AVERAGE(r0!D14,'r1'!D14)</f>
+        <f>AVERAGE(r0!D14,'r1'!D14, 'r2'!D14)</f>
         <v>1</v>
       </c>
       <c r="E14">
-        <f>AVERAGE(r0!E14,'r1'!E14)</f>
+        <f>AVERAGE(r0!E14,'r1'!E14, 'r2'!E14)</f>
         <v>1</v>
       </c>
       <c r="F14">
-        <f>AVERAGE(r0!F14,'r1'!F14)</f>
+        <f>AVERAGE(r0!F14,'r1'!F14, 'r2'!F14)</f>
         <v>1</v>
       </c>
       <c r="G14">
-        <f>AVERAGE(r0!G14,'r1'!G14)</f>
+        <f>AVERAGE(r0!G14,'r1'!G14, 'r2'!G14)</f>
         <v>1</v>
       </c>
       <c r="H14">
-        <f>AVERAGE(r0!H14,'r1'!H14)</f>
+        <f>AVERAGE(r0!H14,'r1'!H14, 'r2'!H14)</f>
         <v>1</v>
       </c>
       <c r="I14">
-        <f>AVERAGE(r0!I14,'r1'!I14)</f>
+        <f>AVERAGE(r0!I14,'r1'!I14, 'r2'!I14)</f>
         <v>2</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B15">
-        <f>AVERAGE(r0!B15,'r1'!B15)</f>
+        <f>AVERAGE(r0!B15,'r1'!B15, 'r2'!B15)</f>
         <v>0</v>
       </c>
       <c r="C15">
-        <f>AVERAGE(r0!C15,'r1'!C15)</f>
+        <f>AVERAGE(r0!C15,'r1'!C15, 'r2'!C15)</f>
         <v>0</v>
       </c>
       <c r="D15">
-        <f>AVERAGE(r0!D15,'r1'!D15)</f>
+        <f>AVERAGE(r0!D15,'r1'!D15, 'r2'!D15)</f>
         <v>0</v>
       </c>
       <c r="E15">
-        <f>AVERAGE(r0!E15,'r1'!E15)</f>
+        <f>AVERAGE(r0!E15,'r1'!E15, 'r2'!E15)</f>
         <v>0</v>
       </c>
       <c r="F15">
-        <f>AVERAGE(r0!F15,'r1'!F15)</f>
+        <f>AVERAGE(r0!F15,'r1'!F15, 'r2'!F15)</f>
         <v>1</v>
       </c>
       <c r="G15">
-        <f>AVERAGE(r0!G15,'r1'!G15)</f>
+        <f>AVERAGE(r0!G15,'r1'!G15, 'r2'!G15)</f>
         <v>0</v>
       </c>
       <c r="H15">
-        <f>AVERAGE(r0!H15,'r1'!H15)</f>
+        <f>AVERAGE(r0!H15,'r1'!H15, 'r2'!H15)</f>
         <v>1</v>
       </c>
       <c r="I15">
-        <f>AVERAGE(r0!I15,'r1'!I15)</f>
+        <f>AVERAGE(r0!I15,'r1'!I15, 'r2'!I15)</f>
         <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B16">
-        <f>AVERAGE(r0!B16,'r1'!B16)</f>
+        <f>AVERAGE(r0!B16,'r1'!B16, 'r2'!B16)</f>
         <v>3</v>
       </c>
       <c r="C16">
-        <f>AVERAGE(r0!C16,'r1'!C16)</f>
+        <f>AVERAGE(r0!C16,'r1'!C16, 'r2'!C16)</f>
         <v>1</v>
       </c>
       <c r="D16">
-        <f>AVERAGE(r0!D16,'r1'!D16)</f>
+        <f>AVERAGE(r0!D16,'r1'!D16, 'r2'!D16)</f>
         <v>1</v>
       </c>
       <c r="E16">
-        <f>AVERAGE(r0!E16,'r1'!E16)</f>
+        <f>AVERAGE(r0!E16,'r1'!E16, 'r2'!E16)</f>
         <v>1</v>
       </c>
       <c r="F16">
-        <f>AVERAGE(r0!F16,'r1'!F16)</f>
+        <f>AVERAGE(r0!F16,'r1'!F16, 'r2'!F16)</f>
         <v>1</v>
       </c>
       <c r="G16">
-        <f>AVERAGE(r0!G16,'r1'!G16)</f>
+        <f>AVERAGE(r0!G16,'r1'!G16, 'r2'!G16)</f>
         <v>1</v>
       </c>
       <c r="H16">
-        <f>AVERAGE(r0!H16,'r1'!H16)</f>
+        <f>AVERAGE(r0!H16,'r1'!H16, 'r2'!H16)</f>
         <v>1</v>
       </c>
       <c r="I16">
-        <f>AVERAGE(r0!I16,'r1'!I16)</f>
+        <f>AVERAGE(r0!I16,'r1'!I16, 'r2'!I16)</f>
         <v>2</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="B17">
-        <f>AVERAGE(r0!B17,'r1'!B17)</f>
+        <f>AVERAGE(r0!B17,'r1'!B17, 'r2'!B17)</f>
         <v>3</v>
       </c>
       <c r="C17">
-        <f>AVERAGE(r0!C17,'r1'!C17)</f>
+        <f>AVERAGE(r0!C17,'r1'!C17, 'r2'!C17)</f>
         <v>1</v>
       </c>
       <c r="D17">
-        <f>AVERAGE(r0!D17,'r1'!D17)</f>
+        <f>AVERAGE(r0!D17,'r1'!D17, 'r2'!D17)</f>
         <v>1</v>
       </c>
       <c r="E17">
-        <f>AVERAGE(r0!E17,'r1'!E17)</f>
+        <f>AVERAGE(r0!E17,'r1'!E17, 'r2'!E17)</f>
         <v>1</v>
       </c>
       <c r="F17">
-        <f>AVERAGE(r0!F17,'r1'!F17)</f>
+        <f>AVERAGE(r0!F17,'r1'!F17, 'r2'!F17)</f>
         <v>1</v>
       </c>
       <c r="G17">
-        <f>AVERAGE(r0!G17,'r1'!G17)</f>
+        <f>AVERAGE(r0!G17,'r1'!G17, 'r2'!G17)</f>
         <v>1</v>
       </c>
       <c r="H17">
-        <f>AVERAGE(r0!H17,'r1'!H17)</f>
+        <f>AVERAGE(r0!H17,'r1'!H17, 'r2'!H17)</f>
         <v>1</v>
       </c>
       <c r="I17">
-        <f>AVERAGE(r0!I17,'r1'!I17)</f>
+        <f>AVERAGE(r0!I17,'r1'!I17, 'r2'!I17)</f>
         <v>2</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B18">
-        <f>AVERAGE(r0!B18,'r1'!B18)</f>
-        <v>0</v>
-      </c>
-      <c r="C18">
-        <f>AVERAGE(r0!C18,'r1'!C18)</f>
-        <v>0</v>
+        <f>AVERAGE(r0!B18,'r1'!B18, 'r2'!B18)</f>
+        <v>1</v>
+      </c>
+      <c r="C18" s="1">
+        <f>AVERAGE(r0!C18,'r1'!C18, 'r2'!C18)</f>
+        <v>0.66666666666666663</v>
       </c>
       <c r="D18">
-        <f>AVERAGE(r0!D18,'r1'!D18)</f>
+        <f>AVERAGE(r0!D18,'r1'!D18, 'r2'!D18)</f>
         <v>0</v>
       </c>
       <c r="E18">
-        <f>AVERAGE(r0!E18,'r1'!E18)</f>
+        <f>AVERAGE(r0!E18,'r1'!E18, 'r2'!E18)</f>
         <v>0</v>
       </c>
       <c r="F18">
-        <f>AVERAGE(r0!F18,'r1'!F18)</f>
+        <f>AVERAGE(r0!F18,'r1'!F18, 'r2'!F18)</f>
         <v>0</v>
       </c>
       <c r="G18">
-        <f>AVERAGE(r0!G18,'r1'!G18)</f>
+        <f>AVERAGE(r0!G18,'r1'!G18, 'r2'!G18)</f>
         <v>0</v>
       </c>
       <c r="H18">
-        <f>AVERAGE(r0!H18,'r1'!H18)</f>
+        <f>AVERAGE(r0!H18,'r1'!H18, 'r2'!H18)</f>
         <v>0</v>
       </c>
       <c r="I18">
-        <f>AVERAGE(r0!I18,'r1'!I18)</f>
+        <f>AVERAGE(r0!I18,'r1'!I18, 'r2'!I18)</f>
         <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B19">
-        <f>AVERAGE(r0!B19,'r1'!B19)</f>
+        <f>AVERAGE(r0!B19,'r1'!B19, 'r2'!B19)</f>
         <v>0</v>
       </c>
       <c r="C19">
-        <f>AVERAGE(r0!C19,'r1'!C19)</f>
+        <f>AVERAGE(r0!C19,'r1'!C19, 'r2'!C19)</f>
         <v>0</v>
       </c>
       <c r="D19">
-        <f>AVERAGE(r0!D19,'r1'!D19)</f>
+        <f>AVERAGE(r0!D19,'r1'!D19, 'r2'!D19)</f>
         <v>0</v>
       </c>
       <c r="E19">
-        <f>AVERAGE(r0!E19,'r1'!E19)</f>
+        <f>AVERAGE(r0!E19,'r1'!E19, 'r2'!E19)</f>
         <v>0</v>
       </c>
       <c r="F19">
-        <f>AVERAGE(r0!F19,'r1'!F19)</f>
+        <f>AVERAGE(r0!F19,'r1'!F19, 'r2'!F19)</f>
         <v>0</v>
       </c>
       <c r="G19">
-        <f>AVERAGE(r0!G19,'r1'!G19)</f>
+        <f>AVERAGE(r0!G19,'r1'!G19, 'r2'!G19)</f>
         <v>0</v>
       </c>
       <c r="H19">
-        <f>AVERAGE(r0!H19,'r1'!H19)</f>
+        <f>AVERAGE(r0!H19,'r1'!H19, 'r2'!H19)</f>
         <v>0</v>
       </c>
       <c r="I19">
-        <f>AVERAGE(r0!I19,'r1'!I19)</f>
+        <f>AVERAGE(r0!I19,'r1'!I19, 'r2'!I19)</f>
         <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B20">
-        <f>AVERAGE(r0!B20,'r1'!B20)</f>
+        <f>AVERAGE(r0!B20,'r1'!B20, 'r2'!B20)</f>
         <v>0</v>
       </c>
       <c r="C20">
-        <f>AVERAGE(r0!C20,'r1'!C20)</f>
-        <v>0</v>
-      </c>
-      <c r="D20">
-        <f>AVERAGE(r0!D20,'r1'!D20)</f>
-        <v>0</v>
+        <f>AVERAGE(r0!C20,'r1'!C20, 'r2'!C20)</f>
+        <v>0</v>
+      </c>
+      <c r="D20" s="1">
+        <f>AVERAGE(r0!D20,'r1'!D20, 'r2'!D20)</f>
+        <v>0.33333333333333331</v>
       </c>
       <c r="E20">
-        <f>AVERAGE(r0!E20,'r1'!E20)</f>
-        <v>0</v>
-      </c>
-      <c r="F20">
-        <f>AVERAGE(r0!F20,'r1'!F20)</f>
-        <v>0.5</v>
-      </c>
-      <c r="G20">
-        <f>AVERAGE(r0!G20,'r1'!G20)</f>
-        <v>1</v>
+        <f>AVERAGE(r0!E20,'r1'!E20, 'r2'!E20)</f>
+        <v>0</v>
+      </c>
+      <c r="F20" s="1">
+        <f>AVERAGE(r0!F20,'r1'!F20, 'r2'!F20)</f>
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="G20" s="1">
+        <f>AVERAGE(r0!G20,'r1'!G20, 'r2'!G20)</f>
+        <v>1.3333333333333333</v>
       </c>
       <c r="H20">
-        <f>AVERAGE(r0!H20,'r1'!H20)</f>
+        <f>AVERAGE(r0!H20,'r1'!H20, 'r2'!H20)</f>
         <v>0</v>
       </c>
       <c r="I20">
-        <f>AVERAGE(r0!I20,'r1'!I20)</f>
+        <f>AVERAGE(r0!I20,'r1'!I20, 'r2'!I20)</f>
         <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B21" s="1">
-        <f>AVERAGE(r0!B21,'r1'!B21)</f>
-        <v>23.100999999999999</v>
+        <f>AVERAGE(r0!B21,'r1'!B21, 'r2'!B21)</f>
+        <v>25.585333333333335</v>
       </c>
       <c r="C21" s="1">
-        <f>AVERAGE(r0!C21,'r1'!C21)</f>
-        <v>22.628</v>
+        <f>AVERAGE(r0!C21,'r1'!C21, 'r2'!C21)</f>
+        <v>21.831333333333333</v>
       </c>
       <c r="D21" s="1">
-        <f>AVERAGE(r0!D21,'r1'!D21)</f>
-        <v>16.874500000000001</v>
+        <f>AVERAGE(r0!D21,'r1'!D21, 'r2'!D21)</f>
+        <v>15.663666666666666</v>
       </c>
       <c r="E21" s="1">
-        <f>AVERAGE(r0!E21,'r1'!E21)</f>
-        <v>17.591999999999999</v>
+        <f>AVERAGE(r0!E21,'r1'!E21, 'r2'!E21)</f>
+        <v>17.267666666666667</v>
       </c>
       <c r="F21" s="1">
-        <f>AVERAGE(r0!F21,'r1'!F21)</f>
-        <v>12.798999999999999</v>
+        <f>AVERAGE(r0!F21,'r1'!F21, 'r2'!F21)</f>
+        <v>12.766666666666666</v>
       </c>
       <c r="G21" s="1">
-        <f>AVERAGE(r0!G21,'r1'!G21)</f>
-        <v>15.265499999999999</v>
+        <f>AVERAGE(r0!G21,'r1'!G21, 'r2'!G21)</f>
+        <v>13.334333333333333</v>
       </c>
       <c r="H21" s="1">
-        <f>AVERAGE(r0!H21,'r1'!H21)</f>
-        <v>20.458500000000001</v>
+        <f>AVERAGE(r0!H21,'r1'!H21, 'r2'!H21)</f>
+        <v>17.989000000000001</v>
       </c>
       <c r="I21" s="1">
-        <f>AVERAGE(r0!I21,'r1'!I21)</f>
-        <v>15.8475</v>
+        <f>AVERAGE(r0!I21,'r1'!I21, 'r2'!I21)</f>
+        <v>15.735666666666667</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>19</v>
+      </c>
+      <c r="B22" s="1">
+        <f>AVERAGE(r0!B22,'r1'!B22, 'r2'!B22)</f>
+        <v>2.4386666666666668E-2</v>
+      </c>
+      <c r="C22" s="1">
+        <f>AVERAGE(r0!C22,'r1'!C22, 'r2'!C22)</f>
+        <v>2.2651000000000001E-2</v>
+      </c>
+      <c r="D22" s="1">
+        <f>AVERAGE(r0!D22,'r1'!D22, 'r2'!D22)</f>
+        <v>1.8483666666666666E-2</v>
+      </c>
+      <c r="E22" s="1">
+        <f>AVERAGE(r0!E22,'r1'!E22, 'r2'!E22)</f>
+        <v>2.0503E-2</v>
+      </c>
+      <c r="F22" s="1">
+        <f>AVERAGE(r0!F22,'r1'!F22, 'r2'!F22)</f>
+        <v>1.6129333333333332E-2</v>
+      </c>
+      <c r="G22" s="1">
+        <f>AVERAGE(r0!G22,'r1'!G22, 'r2'!G22)</f>
+        <v>1.4313666666666664E-2</v>
+      </c>
+      <c r="H22" s="1">
+        <f>AVERAGE(r0!H22,'r1'!H22, 'r2'!H22)</f>
+        <v>1.5993333333333335E-2</v>
+      </c>
+      <c r="I22" s="1">
+        <f>AVERAGE(r0!I22,'r1'!I22, 'r2'!I22)</f>
+        <v>1.7988666666666667E-2</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
@@ -2876,7 +3584,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE3232CA-EC8E-404A-B90B-03381B7790AE}">
   <dimension ref="A1:I23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2888,101 +3596,101 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>49</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>52</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>58</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>59</v>
+        <v>47</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>61</v>
+        <v>49</v>
       </c>
     </row>
     <row r="21" spans="2:9" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
added r3 results data
</commit_message>
<xml_diff>
--- a/finalReport.xlsx
+++ b/finalReport.xlsx
@@ -8,16 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fedev\Documents\UNICAM\Phd\unmock\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B5B9E6A-A321-4164-858C-8673DDB1DAD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{418FE2C4-8FE5-4F13-B2DB-BAF1A1C20EBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A0F7C0B4-A897-4B1D-9E87-712A814F4D93}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{A0F7C0B4-A897-4B1D-9E87-712A814F4D93}"/>
   </bookViews>
   <sheets>
     <sheet name="r0" sheetId="1" r:id="rId1"/>
     <sheet name="r1" sheetId="2" r:id="rId2"/>
     <sheet name="r2" sheetId="5" r:id="rId3"/>
-    <sheet name="global" sheetId="4" r:id="rId4"/>
-    <sheet name="Test IDs" sheetId="3" r:id="rId5"/>
+    <sheet name="r3" sheetId="6" r:id="rId4"/>
+    <sheet name="global" sheetId="4" r:id="rId5"/>
+    <sheet name="Test IDs" sheetId="3" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="56">
   <si>
     <t>Target test</t>
   </si>
@@ -205,6 +206,12 @@
   </si>
   <si>
     <t>Transformed argument matcher in stub with semantic errors</t>
+  </si>
+  <si>
+    <t>Approximated Cost ($)</t>
+  </si>
+  <si>
+    <t>Approximated Generation time (sec)</t>
   </si>
 </sst>
 </file>
@@ -2748,12 +2755,580 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84C92F30-4B94-47F9-B1CE-35111BB21FA9}">
+  <dimension ref="A1:I24"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="55.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="9" width="11.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="str">
+        <f>'Test IDs'!C2</f>
+        <v>DS.1</v>
+      </c>
+      <c r="C1" t="str">
+        <f>'Test IDs'!C3</f>
+        <v>DS.2</v>
+      </c>
+      <c r="D1" t="str">
+        <f>'Test IDs'!C4</f>
+        <v>DS.3</v>
+      </c>
+      <c r="E1" t="str">
+        <f>'Test IDs'!C5</f>
+        <v>DS.4</v>
+      </c>
+      <c r="F1" t="str">
+        <f>'Test IDs'!C6</f>
+        <v>N.1</v>
+      </c>
+      <c r="G1" t="str">
+        <f>'Test IDs'!C7</f>
+        <v>N.2</v>
+      </c>
+      <c r="H1" t="str">
+        <f>'Test IDs'!C8</f>
+        <v>N.3</v>
+      </c>
+      <c r="I1" t="str">
+        <f>'Test IDs'!C9</f>
+        <v>N.4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>3</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6">
+        <v>1</v>
+      </c>
+      <c r="I6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>0</v>
+      </c>
+      <c r="C7">
+        <v>2</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>0</v>
+      </c>
+      <c r="C8">
+        <v>0</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>0</v>
+      </c>
+      <c r="C9">
+        <v>0</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="F9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>50</v>
+      </c>
+      <c r="B10">
+        <v>0</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <v>0</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <v>0</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>51</v>
+      </c>
+      <c r="B11">
+        <v>0</v>
+      </c>
+      <c r="C11">
+        <v>0</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11">
+        <v>0</v>
+      </c>
+      <c r="F11">
+        <v>0</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11">
+        <v>0</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>52</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12">
+        <v>0</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="F12">
+        <v>0</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="I12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>53</v>
+      </c>
+      <c r="B13">
+        <v>0</v>
+      </c>
+      <c r="C13">
+        <v>1</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+      <c r="F13">
+        <v>0</v>
+      </c>
+      <c r="G13">
+        <v>0</v>
+      </c>
+      <c r="H13">
+        <v>0</v>
+      </c>
+      <c r="I13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>9</v>
+      </c>
+      <c r="B14">
+        <v>3</v>
+      </c>
+      <c r="C14">
+        <v>1</v>
+      </c>
+      <c r="D14">
+        <v>1</v>
+      </c>
+      <c r="E14">
+        <v>1</v>
+      </c>
+      <c r="F14">
+        <v>1</v>
+      </c>
+      <c r="G14">
+        <v>1</v>
+      </c>
+      <c r="H14">
+        <v>1</v>
+      </c>
+      <c r="I14">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>10</v>
+      </c>
+      <c r="B15">
+        <v>0</v>
+      </c>
+      <c r="C15">
+        <v>0</v>
+      </c>
+      <c r="D15">
+        <v>0</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+      <c r="F15">
+        <v>1</v>
+      </c>
+      <c r="G15">
+        <v>0</v>
+      </c>
+      <c r="H15">
+        <v>1</v>
+      </c>
+      <c r="I15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>11</v>
+      </c>
+      <c r="B16">
+        <v>3</v>
+      </c>
+      <c r="C16">
+        <v>1</v>
+      </c>
+      <c r="D16">
+        <v>1</v>
+      </c>
+      <c r="E16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>12</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17">
+        <v>1</v>
+      </c>
+      <c r="D17">
+        <v>1</v>
+      </c>
+      <c r="E17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>13</v>
+      </c>
+      <c r="B18">
+        <v>0</v>
+      </c>
+      <c r="C18">
+        <v>0</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>14</v>
+      </c>
+      <c r="B19">
+        <v>0</v>
+      </c>
+      <c r="C19">
+        <v>0</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>15</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20">
+        <v>0</v>
+      </c>
+      <c r="D20">
+        <v>1</v>
+      </c>
+      <c r="E20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>16</v>
+      </c>
+      <c r="B21" s="1">
+        <v>24.46</v>
+      </c>
+      <c r="C21" s="1">
+        <v>20.010999999999999</v>
+      </c>
+      <c r="D21" s="1">
+        <v>14.097</v>
+      </c>
+      <c r="E21" s="1">
+        <v>19.84</v>
+      </c>
+      <c r="F21" s="1"/>
+      <c r="G21" s="1"/>
+      <c r="H21" s="1"/>
+      <c r="I21" s="1"/>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>19</v>
+      </c>
+      <c r="B22" s="1">
+        <v>2.3654000000000001E-2</v>
+      </c>
+      <c r="C22" s="1">
+        <v>2.3720000000000001E-2</v>
+      </c>
+      <c r="D22" s="1">
+        <v>1.3103E-2</v>
+      </c>
+      <c r="E22" s="1">
+        <v>1.8454999999999999E-2</v>
+      </c>
+      <c r="F22" s="1"/>
+      <c r="G22" s="1"/>
+      <c r="H22" s="1"/>
+      <c r="I22" s="1"/>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>17</v>
+      </c>
+      <c r="B23" t="s">
+        <v>18</v>
+      </c>
+      <c r="C23" t="s">
+        <v>18</v>
+      </c>
+      <c r="D23" t="s">
+        <v>18</v>
+      </c>
+      <c r="E23" t="s">
+        <v>18</v>
+      </c>
+      <c r="F23" t="s">
+        <v>18</v>
+      </c>
+      <c r="G23" t="s">
+        <v>18</v>
+      </c>
+      <c r="H23" t="s">
+        <v>18</v>
+      </c>
+      <c r="I23" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>20</v>
+      </c>
+      <c r="B24" t="s">
+        <v>21</v>
+      </c>
+      <c r="C24" t="s">
+        <v>22</v>
+      </c>
+      <c r="D24" t="s">
+        <v>22</v>
+      </c>
+      <c r="E24" t="s">
+        <v>21</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E040BF79-8B7D-43C4-816A-164CB83CAB3E}">
   <dimension ref="A1:I23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="61.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="9" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.85546875" customWidth="1"/>
+    <col min="3" max="9" width="11.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2798,35 +3373,35 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <f>AVERAGE(r0!B2,'r1'!B2, 'r2'!B2)</f>
+        <f>AVERAGE(r0!B2,'r1'!B2, 'r2'!B2, 'r3'!B2)</f>
         <v>3</v>
       </c>
       <c r="C2">
-        <f>AVERAGE(r0!C2,'r1'!C2, 'r2'!C2)</f>
+        <f>AVERAGE(r0!C2,'r1'!C2, 'r2'!C2, 'r3'!C2)</f>
         <v>2</v>
       </c>
       <c r="D2">
-        <f>AVERAGE(r0!D2,'r1'!D2, 'r2'!D2)</f>
+        <f>AVERAGE(r0!D2,'r1'!D2, 'r2'!D2, 'r3'!D2)</f>
         <v>1</v>
       </c>
       <c r="E2">
-        <f>AVERAGE(r0!E2,'r1'!E2, 'r2'!E2)</f>
+        <f>AVERAGE(r0!E2,'r1'!E2, 'r2'!E2, 'r3'!E2)</f>
         <v>1</v>
       </c>
       <c r="F2">
-        <f>AVERAGE(r0!F2,'r1'!F2, 'r2'!F2)</f>
+        <f>AVERAGE(r0!F2,'r1'!F2, 'r2'!F2, 'r3'!F2)</f>
         <v>1</v>
       </c>
       <c r="G2">
-        <f>AVERAGE(r0!G2,'r1'!G2, 'r2'!G2)</f>
+        <f>AVERAGE(r0!G2,'r1'!G2, 'r2'!G2, 'r3'!G2)</f>
         <v>0</v>
       </c>
       <c r="H2">
-        <f>AVERAGE(r0!H2,'r1'!H2, 'r2'!H2)</f>
+        <f>AVERAGE(r0!H2,'r1'!H2, 'r2'!H2, 'r3'!H2)</f>
         <v>0</v>
       </c>
       <c r="I2">
-        <f>AVERAGE(r0!I2,'r1'!I2, 'r2'!I2)</f>
+        <f>AVERAGE(r0!I2,'r1'!I2, 'r2'!I2, 'r3'!I2)</f>
         <v>1</v>
       </c>
     </row>
@@ -2835,35 +3410,35 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <f>AVERAGE(r0!B3,'r1'!B3, 'r2'!B3)</f>
+        <f>AVERAGE(r0!B3,'r1'!B3, 'r2'!B3, 'r3'!B3)</f>
         <v>3</v>
       </c>
       <c r="C3">
-        <f>AVERAGE(r0!C3,'r1'!C3, 'r2'!C3)</f>
+        <f>AVERAGE(r0!C3,'r1'!C3, 'r2'!C3, 'r3'!C3)</f>
         <v>2</v>
       </c>
       <c r="D3">
-        <f>AVERAGE(r0!D3,'r1'!D3, 'r2'!D3)</f>
+        <f>AVERAGE(r0!D3,'r1'!D3, 'r2'!D3, 'r3'!D3)</f>
         <v>1</v>
       </c>
       <c r="E3">
-        <f>AVERAGE(r0!E3,'r1'!E3, 'r2'!E3)</f>
+        <f>AVERAGE(r0!E3,'r1'!E3, 'r2'!E3, 'r3'!E3)</f>
         <v>1</v>
       </c>
       <c r="F3">
-        <f>AVERAGE(r0!F3,'r1'!F3, 'r2'!F3)</f>
+        <f>AVERAGE(r0!F3,'r1'!F3, 'r2'!F3, 'r3'!F3)</f>
         <v>1</v>
       </c>
       <c r="G3">
-        <f>AVERAGE(r0!G3,'r1'!G3, 'r2'!G3)</f>
+        <f>AVERAGE(r0!G3,'r1'!G3, 'r2'!G3, 'r3'!G3)</f>
         <v>0</v>
       </c>
       <c r="H3">
-        <f>AVERAGE(r0!H3,'r1'!H3, 'r2'!H3)</f>
+        <f>AVERAGE(r0!H3,'r1'!H3, 'r2'!H3, 'r3'!H3)</f>
         <v>0</v>
       </c>
       <c r="I3">
-        <f>AVERAGE(r0!I3,'r1'!I3, 'r2'!I3)</f>
+        <f>AVERAGE(r0!I3,'r1'!I3, 'r2'!I3, 'r3'!I3)</f>
         <v>1</v>
       </c>
     </row>
@@ -2872,35 +3447,35 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <f>AVERAGE(r0!B4,'r1'!B4, 'r2'!B4)</f>
+        <f>AVERAGE(r0!B4,'r1'!B4, 'r2'!B4, 'r3'!B4)</f>
         <v>0</v>
       </c>
       <c r="C4">
-        <f>AVERAGE(r0!C4,'r1'!C4, 'r2'!C4)</f>
+        <f>AVERAGE(r0!C4,'r1'!C4, 'r2'!C4, 'r3'!C4)</f>
         <v>0</v>
       </c>
       <c r="D4">
-        <f>AVERAGE(r0!D4,'r1'!D4, 'r2'!D4)</f>
+        <f>AVERAGE(r0!D4,'r1'!D4, 'r2'!D4, 'r3'!D4)</f>
         <v>0</v>
       </c>
       <c r="E4">
-        <f>AVERAGE(r0!E4,'r1'!E4, 'r2'!E4)</f>
+        <f>AVERAGE(r0!E4,'r1'!E4, 'r2'!E4, 'r3'!E4)</f>
         <v>0</v>
       </c>
       <c r="F4">
-        <f>AVERAGE(r0!F4,'r1'!F4, 'r2'!F4)</f>
+        <f>AVERAGE(r0!F4,'r1'!F4, 'r2'!F4, 'r3'!F4)</f>
         <v>0</v>
       </c>
       <c r="G4">
-        <f>AVERAGE(r0!G4,'r1'!G4, 'r2'!G4)</f>
+        <f>AVERAGE(r0!G4,'r1'!G4, 'r2'!G4, 'r3'!G4)</f>
         <v>0</v>
       </c>
       <c r="H4">
-        <f>AVERAGE(r0!H4,'r1'!H4, 'r2'!H4)</f>
+        <f>AVERAGE(r0!H4,'r1'!H4, 'r2'!H4, 'r3'!H4)</f>
         <v>0</v>
       </c>
       <c r="I4">
-        <f>AVERAGE(r0!I4,'r1'!I4, 'r2'!I4)</f>
+        <f>AVERAGE(r0!I4,'r1'!I4, 'r2'!I4, 'r3'!I4)</f>
         <v>0</v>
       </c>
     </row>
@@ -2909,35 +3484,35 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <f>AVERAGE(r0!B5,'r1'!B5, 'r2'!B5)</f>
-        <v>1</v>
-      </c>
-      <c r="C5" s="1">
-        <f>AVERAGE(r0!C5,'r1'!C5, 'r2'!C5)</f>
-        <v>0.33333333333333331</v>
+        <f>AVERAGE(r0!B5,'r1'!B5, 'r2'!B5, 'r3'!B5)</f>
+        <v>0.75</v>
+      </c>
+      <c r="C5">
+        <f>AVERAGE(r0!C5,'r1'!C5, 'r2'!C5, 'r3'!C5)</f>
+        <v>0.25</v>
       </c>
       <c r="D5">
-        <f>AVERAGE(r0!D5,'r1'!D5, 'r2'!D5)</f>
+        <f>AVERAGE(r0!D5,'r1'!D5, 'r2'!D5, 'r3'!D5)</f>
         <v>0</v>
       </c>
       <c r="E5">
-        <f>AVERAGE(r0!E5,'r1'!E5, 'r2'!E5)</f>
+        <f>AVERAGE(r0!E5,'r1'!E5, 'r2'!E5, 'r3'!E5)</f>
         <v>0</v>
       </c>
       <c r="F5">
-        <f>AVERAGE(r0!F5,'r1'!F5, 'r2'!F5)</f>
+        <f>AVERAGE(r0!F5,'r1'!F5, 'r2'!F5, 'r3'!F5)</f>
         <v>0</v>
       </c>
       <c r="G5">
-        <f>AVERAGE(r0!G5,'r1'!G5, 'r2'!G5)</f>
+        <f>AVERAGE(r0!G5,'r1'!G5, 'r2'!G5, 'r3'!G5)</f>
         <v>0</v>
       </c>
       <c r="H5">
-        <f>AVERAGE(r0!H5,'r1'!H5, 'r2'!H5)</f>
+        <f>AVERAGE(r0!H5,'r1'!H5, 'r2'!H5, 'r3'!H5)</f>
         <v>0</v>
       </c>
       <c r="I5">
-        <f>AVERAGE(r0!I5,'r1'!I5, 'r2'!I5)</f>
+        <f>AVERAGE(r0!I5,'r1'!I5, 'r2'!I5, 'r3'!I5)</f>
         <v>0</v>
       </c>
     </row>
@@ -2946,35 +3521,35 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <f>AVERAGE(r0!B6,'r1'!B6, 'r2'!B6)</f>
+        <f>AVERAGE(r0!B6,'r1'!B6, 'r2'!B6, 'r3'!B6)</f>
         <v>0</v>
       </c>
       <c r="C6">
-        <f>AVERAGE(r0!C6,'r1'!C6, 'r2'!C6)</f>
+        <f>AVERAGE(r0!C6,'r1'!C6, 'r2'!C6, 'r3'!C6)</f>
         <v>2</v>
       </c>
       <c r="D6">
-        <f>AVERAGE(r0!D6,'r1'!D6, 'r2'!D6)</f>
+        <f>AVERAGE(r0!D6,'r1'!D6, 'r2'!D6, 'r3'!D6)</f>
         <v>0</v>
       </c>
       <c r="E6">
-        <f>AVERAGE(r0!E6,'r1'!E6, 'r2'!E6)</f>
+        <f>AVERAGE(r0!E6,'r1'!E6, 'r2'!E6, 'r3'!E6)</f>
         <v>0</v>
       </c>
       <c r="F6">
-        <f>AVERAGE(r0!F6,'r1'!F6, 'r2'!F6)</f>
+        <f>AVERAGE(r0!F6,'r1'!F6, 'r2'!F6, 'r3'!F6)</f>
         <v>0</v>
       </c>
       <c r="G6">
-        <f>AVERAGE(r0!G6,'r1'!G6, 'r2'!G6)</f>
+        <f>AVERAGE(r0!G6,'r1'!G6, 'r2'!G6, 'r3'!G6)</f>
         <v>1</v>
       </c>
       <c r="H6">
-        <f>AVERAGE(r0!H6,'r1'!H6, 'r2'!H6)</f>
+        <f>AVERAGE(r0!H6,'r1'!H6, 'r2'!H6, 'r3'!H6)</f>
         <v>1</v>
       </c>
       <c r="I6">
-        <f>AVERAGE(r0!I6,'r1'!I6, 'r2'!I6)</f>
+        <f>AVERAGE(r0!I6,'r1'!I6, 'r2'!I6, 'r3'!I6)</f>
         <v>1</v>
       </c>
     </row>
@@ -2983,35 +3558,35 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <f>AVERAGE(r0!B7,'r1'!B7, 'r2'!B7)</f>
+        <f>AVERAGE(r0!B7,'r1'!B7, 'r2'!B7, 'r3'!B7)</f>
         <v>0</v>
       </c>
       <c r="C7">
-        <f>AVERAGE(r0!C7,'r1'!C7, 'r2'!C7)</f>
+        <f>AVERAGE(r0!C7,'r1'!C7, 'r2'!C7, 'r3'!C7)</f>
         <v>2</v>
       </c>
       <c r="D7">
-        <f>AVERAGE(r0!D7,'r1'!D7, 'r2'!D7)</f>
+        <f>AVERAGE(r0!D7,'r1'!D7, 'r2'!D7, 'r3'!D7)</f>
         <v>0</v>
       </c>
       <c r="E7">
-        <f>AVERAGE(r0!E7,'r1'!E7, 'r2'!E7)</f>
+        <f>AVERAGE(r0!E7,'r1'!E7, 'r2'!E7, 'r3'!E7)</f>
         <v>0</v>
       </c>
       <c r="F7">
-        <f>AVERAGE(r0!F7,'r1'!F7, 'r2'!F7)</f>
+        <f>AVERAGE(r0!F7,'r1'!F7, 'r2'!F7, 'r3'!F7)</f>
         <v>0</v>
       </c>
       <c r="G7">
-        <f>AVERAGE(r0!G7,'r1'!G7, 'r2'!G7)</f>
-        <v>1</v>
-      </c>
-      <c r="H7" s="1">
-        <f>AVERAGE(r0!H7,'r1'!H7, 'r2'!H7)</f>
+        <f>AVERAGE(r0!G7,'r1'!G7, 'r2'!G7, 'r3'!G7)</f>
+        <v>1</v>
+      </c>
+      <c r="H7">
+        <f>AVERAGE(r0!H7,'r1'!H7, 'r2'!H7, 'r3'!H7)</f>
         <v>0.66666666666666663</v>
       </c>
       <c r="I7">
-        <f>AVERAGE(r0!I7,'r1'!I7, 'r2'!I7)</f>
+        <f>AVERAGE(r0!I7,'r1'!I7, 'r2'!I7, 'r3'!I7)</f>
         <v>1</v>
       </c>
     </row>
@@ -3020,35 +3595,35 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <f>AVERAGE(r0!B8,'r1'!B8, 'r2'!B8)</f>
+        <f>AVERAGE(r0!B8,'r1'!B8, 'r2'!B8, 'r3'!B8)</f>
         <v>0</v>
       </c>
       <c r="C8">
-        <f>AVERAGE(r0!C8,'r1'!C8, 'r2'!C8)</f>
+        <f>AVERAGE(r0!C8,'r1'!C8, 'r2'!C8, 'r3'!C8)</f>
         <v>0</v>
       </c>
       <c r="D8">
-        <f>AVERAGE(r0!D8,'r1'!D8, 'r2'!D8)</f>
+        <f>AVERAGE(r0!D8,'r1'!D8, 'r2'!D8, 'r3'!D8)</f>
         <v>0</v>
       </c>
       <c r="E8">
-        <f>AVERAGE(r0!E8,'r1'!E8, 'r2'!E8)</f>
+        <f>AVERAGE(r0!E8,'r1'!E8, 'r2'!E8, 'r3'!E8)</f>
         <v>0</v>
       </c>
       <c r="F8">
-        <f>AVERAGE(r0!F8,'r1'!F8, 'r2'!F8)</f>
-        <v>0</v>
-      </c>
-      <c r="G8" s="1">
-        <f>AVERAGE(r0!G8,'r1'!G8, 'r2'!G8)</f>
+        <f>AVERAGE(r0!F8,'r1'!F8, 'r2'!F8, 'r3'!F8)</f>
+        <v>0</v>
+      </c>
+      <c r="G8">
+        <f>AVERAGE(r0!G8,'r1'!G8, 'r2'!G8, 'r3'!G8)</f>
         <v>0.33333333333333331</v>
       </c>
-      <c r="H8" s="1">
-        <f>AVERAGE(r0!H8,'r1'!H8, 'r2'!H8)</f>
+      <c r="H8">
+        <f>AVERAGE(r0!H8,'r1'!H8, 'r2'!H8, 'r3'!H8)</f>
         <v>0.33333333333333331</v>
       </c>
       <c r="I8">
-        <f>AVERAGE(r0!I8,'r1'!I8, 'r2'!I8)</f>
+        <f>AVERAGE(r0!I8,'r1'!I8, 'r2'!I8, 'r3'!I8)</f>
         <v>0</v>
       </c>
     </row>
@@ -3057,35 +3632,35 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <f>AVERAGE(r0!B9,'r1'!B9, 'r2'!B9)</f>
+        <f>AVERAGE(r0!B9,'r1'!B9, 'r2'!B9, 'r3'!B9)</f>
         <v>0</v>
       </c>
       <c r="C9">
-        <f>AVERAGE(r0!C9,'r1'!C9, 'r2'!C9)</f>
+        <f>AVERAGE(r0!C9,'r1'!C9, 'r2'!C9, 'r3'!C9)</f>
         <v>0</v>
       </c>
       <c r="D9">
-        <f>AVERAGE(r0!D9,'r1'!D9, 'r2'!D9)</f>
+        <f>AVERAGE(r0!D9,'r1'!D9, 'r2'!D9, 'r3'!D9)</f>
         <v>0</v>
       </c>
       <c r="E9">
-        <f>AVERAGE(r0!E9,'r1'!E9, 'r2'!E9)</f>
+        <f>AVERAGE(r0!E9,'r1'!E9, 'r2'!E9, 'r3'!E9)</f>
         <v>0</v>
       </c>
       <c r="F9">
-        <f>AVERAGE(r0!F9,'r1'!F9, 'r2'!F9)</f>
+        <f>AVERAGE(r0!F9,'r1'!F9, 'r2'!F9, 'r3'!F9)</f>
         <v>0</v>
       </c>
       <c r="G9">
-        <f>AVERAGE(r0!G9,'r1'!G9, 'r2'!G9)</f>
+        <f>AVERAGE(r0!G9,'r1'!G9, 'r2'!G9, 'r3'!G9)</f>
         <v>0</v>
       </c>
       <c r="H9">
-        <f>AVERAGE(r0!H9,'r1'!H9, 'r2'!H9)</f>
+        <f>AVERAGE(r0!H9,'r1'!H9, 'r2'!H9, 'r3'!H9)</f>
         <v>0</v>
       </c>
       <c r="I9">
-        <f>AVERAGE(r0!I9,'r1'!I9, 'r2'!I9)</f>
+        <f>AVERAGE(r0!I9,'r1'!I9, 'r2'!I9, 'r3'!I9)</f>
         <v>0</v>
       </c>
     </row>
@@ -3094,35 +3669,35 @@
         <v>50</v>
       </c>
       <c r="B10">
-        <f>AVERAGE(r0!B10,'r1'!B10, 'r2'!B10)</f>
+        <f>AVERAGE(r0!B10,'r1'!B10, 'r2'!B10, 'r3'!B10)</f>
         <v>0</v>
       </c>
       <c r="C10">
-        <f>AVERAGE(r0!C10,'r1'!C10, 'r2'!C10)</f>
+        <f>AVERAGE(r0!C10,'r1'!C10, 'r2'!C10, 'r3'!C10)</f>
         <v>1</v>
       </c>
       <c r="D10">
-        <f>AVERAGE(r0!D10,'r1'!D10, 'r2'!D10)</f>
+        <f>AVERAGE(r0!D10,'r1'!D10, 'r2'!D10, 'r3'!D10)</f>
         <v>0</v>
       </c>
       <c r="E10">
-        <f>AVERAGE(r0!E10,'r1'!E10, 'r2'!E10)</f>
+        <f>AVERAGE(r0!E10,'r1'!E10, 'r2'!E10, 'r3'!E10)</f>
         <v>0</v>
       </c>
       <c r="F10">
-        <f>AVERAGE(r0!F10,'r1'!F10, 'r2'!F10)</f>
+        <f>AVERAGE(r0!F10,'r1'!F10, 'r2'!F10, 'r3'!F10)</f>
         <v>0</v>
       </c>
       <c r="G10">
-        <f>AVERAGE(r0!G10,'r1'!G10, 'r2'!G10)</f>
+        <f>AVERAGE(r0!G10,'r1'!G10, 'r2'!G10, 'r3'!G10)</f>
         <v>0</v>
       </c>
       <c r="H10">
-        <f>AVERAGE(r0!H10,'r1'!H10, 'r2'!H10)</f>
+        <f>AVERAGE(r0!H10,'r1'!H10, 'r2'!H10, 'r3'!H10)</f>
         <v>0</v>
       </c>
       <c r="I10">
-        <f>AVERAGE(r0!I10,'r1'!I10, 'r2'!I10)</f>
+        <f>AVERAGE(r0!I10,'r1'!I10, 'r2'!I10, 'r3'!I10)</f>
         <v>0</v>
       </c>
     </row>
@@ -3131,35 +3706,35 @@
         <v>51</v>
       </c>
       <c r="B11">
-        <f>AVERAGE(r0!B11,'r1'!B11, 'r2'!B11)</f>
-        <v>0</v>
-      </c>
-      <c r="C11" s="1">
-        <f>AVERAGE(r0!C11,'r1'!C11, 'r2'!C11)</f>
-        <v>0.66666666666666663</v>
+        <f>AVERAGE(r0!B11,'r1'!B11, 'r2'!B11, 'r3'!B11)</f>
+        <v>0</v>
+      </c>
+      <c r="C11">
+        <f>AVERAGE(r0!C11,'r1'!C11, 'r2'!C11, 'r3'!C11)</f>
+        <v>0.5</v>
       </c>
       <c r="D11">
-        <f>AVERAGE(r0!D11,'r1'!D11, 'r2'!D11)</f>
+        <f>AVERAGE(r0!D11,'r1'!D11, 'r2'!D11, 'r3'!D11)</f>
         <v>0</v>
       </c>
       <c r="E11">
-        <f>AVERAGE(r0!E11,'r1'!E11, 'r2'!E11)</f>
+        <f>AVERAGE(r0!E11,'r1'!E11, 'r2'!E11, 'r3'!E11)</f>
         <v>0</v>
       </c>
       <c r="F11">
-        <f>AVERAGE(r0!F11,'r1'!F11, 'r2'!F11)</f>
+        <f>AVERAGE(r0!F11,'r1'!F11, 'r2'!F11, 'r3'!F11)</f>
         <v>0</v>
       </c>
       <c r="G11">
-        <f>AVERAGE(r0!G11,'r1'!G11, 'r2'!G11)</f>
+        <f>AVERAGE(r0!G11,'r1'!G11, 'r2'!G11, 'r3'!G11)</f>
         <v>0</v>
       </c>
       <c r="H11">
-        <f>AVERAGE(r0!H11,'r1'!H11, 'r2'!H11)</f>
+        <f>AVERAGE(r0!H11,'r1'!H11, 'r2'!H11, 'r3'!H11)</f>
         <v>0</v>
       </c>
       <c r="I11">
-        <f>AVERAGE(r0!I11,'r1'!I11, 'r2'!I11)</f>
+        <f>AVERAGE(r0!I11,'r1'!I11, 'r2'!I11, 'r3'!I11)</f>
         <v>0</v>
       </c>
     </row>
@@ -3168,35 +3743,35 @@
         <v>52</v>
       </c>
       <c r="B12">
-        <f>AVERAGE(r0!B12,'r1'!B12, 'r2'!B12)</f>
+        <f>AVERAGE(r0!B12,'r1'!B12, 'r2'!B12, 'r3'!B12)</f>
         <v>0</v>
       </c>
       <c r="C12">
-        <f>AVERAGE(r0!C12,'r1'!C12, 'r2'!C12)</f>
+        <f>AVERAGE(r0!C12,'r1'!C12, 'r2'!C12, 'r3'!C12)</f>
         <v>0</v>
       </c>
       <c r="D12">
-        <f>AVERAGE(r0!D12,'r1'!D12, 'r2'!D12)</f>
+        <f>AVERAGE(r0!D12,'r1'!D12, 'r2'!D12, 'r3'!D12)</f>
         <v>0</v>
       </c>
       <c r="E12">
-        <f>AVERAGE(r0!E12,'r1'!E12, 'r2'!E12)</f>
+        <f>AVERAGE(r0!E12,'r1'!E12, 'r2'!E12, 'r3'!E12)</f>
         <v>0</v>
       </c>
       <c r="F12">
-        <f>AVERAGE(r0!F12,'r1'!F12, 'r2'!F12)</f>
+        <f>AVERAGE(r0!F12,'r1'!F12, 'r2'!F12, 'r3'!F12)</f>
         <v>0</v>
       </c>
       <c r="G12">
-        <f>AVERAGE(r0!G12,'r1'!G12, 'r2'!G12)</f>
+        <f>AVERAGE(r0!G12,'r1'!G12, 'r2'!G12, 'r3'!G12)</f>
         <v>0</v>
       </c>
       <c r="H12">
-        <f>AVERAGE(r0!H12,'r1'!H12, 'r2'!H12)</f>
+        <f>AVERAGE(r0!H12,'r1'!H12, 'r2'!H12, 'r3'!H12)</f>
         <v>0</v>
       </c>
       <c r="I12">
-        <f>AVERAGE(r0!I12,'r1'!I12, 'r2'!I12)</f>
+        <f>AVERAGE(r0!I12,'r1'!I12, 'r2'!I12, 'r3'!I12)</f>
         <v>0</v>
       </c>
     </row>
@@ -3205,35 +3780,35 @@
         <v>53</v>
       </c>
       <c r="B13">
-        <f>AVERAGE(r0!B13,'r1'!B13, 'r2'!B13)</f>
-        <v>0</v>
-      </c>
-      <c r="C13" s="1">
-        <f>AVERAGE(r0!C13,'r1'!C13, 'r2'!C13)</f>
-        <v>0.33333333333333331</v>
+        <f>AVERAGE(r0!B13,'r1'!B13, 'r2'!B13, 'r3'!B13)</f>
+        <v>0</v>
+      </c>
+      <c r="C13">
+        <f>AVERAGE(r0!C13,'r1'!C13, 'r2'!C13, 'r3'!C13)</f>
+        <v>0.5</v>
       </c>
       <c r="D13">
-        <f>AVERAGE(r0!D13,'r1'!D13, 'r2'!D13)</f>
+        <f>AVERAGE(r0!D13,'r1'!D13, 'r2'!D13, 'r3'!D13)</f>
         <v>0</v>
       </c>
       <c r="E13">
-        <f>AVERAGE(r0!E13,'r1'!E13, 'r2'!E13)</f>
+        <f>AVERAGE(r0!E13,'r1'!E13, 'r2'!E13, 'r3'!E13)</f>
         <v>0</v>
       </c>
       <c r="F13">
-        <f>AVERAGE(r0!F13,'r1'!F13, 'r2'!F13)</f>
+        <f>AVERAGE(r0!F13,'r1'!F13, 'r2'!F13, 'r3'!F13)</f>
         <v>0</v>
       </c>
       <c r="G13">
-        <f>AVERAGE(r0!G13,'r1'!G13, 'r2'!G13)</f>
+        <f>AVERAGE(r0!G13,'r1'!G13, 'r2'!G13, 'r3'!G13)</f>
         <v>0</v>
       </c>
       <c r="H13">
-        <f>AVERAGE(r0!H13,'r1'!H13, 'r2'!H13)</f>
+        <f>AVERAGE(r0!H13,'r1'!H13, 'r2'!H13, 'r3'!H13)</f>
         <v>0</v>
       </c>
       <c r="I13">
-        <f>AVERAGE(r0!I13,'r1'!I13, 'r2'!I13)</f>
+        <f>AVERAGE(r0!I13,'r1'!I13, 'r2'!I13, 'r3'!I13)</f>
         <v>0</v>
       </c>
     </row>
@@ -3242,35 +3817,35 @@
         <v>9</v>
       </c>
       <c r="B14">
-        <f>AVERAGE(r0!B14,'r1'!B14, 'r2'!B14)</f>
+        <f>AVERAGE(r0!B14,'r1'!B14, 'r2'!B14, 'r3'!B14)</f>
         <v>3</v>
       </c>
       <c r="C14">
-        <f>AVERAGE(r0!C14,'r1'!C14, 'r2'!C14)</f>
+        <f>AVERAGE(r0!C14,'r1'!C14, 'r2'!C14, 'r3'!C14)</f>
         <v>1</v>
       </c>
       <c r="D14">
-        <f>AVERAGE(r0!D14,'r1'!D14, 'r2'!D14)</f>
+        <f>AVERAGE(r0!D14,'r1'!D14, 'r2'!D14, 'r3'!D14)</f>
         <v>1</v>
       </c>
       <c r="E14">
-        <f>AVERAGE(r0!E14,'r1'!E14, 'r2'!E14)</f>
+        <f>AVERAGE(r0!E14,'r1'!E14, 'r2'!E14, 'r3'!E14)</f>
         <v>1</v>
       </c>
       <c r="F14">
-        <f>AVERAGE(r0!F14,'r1'!F14, 'r2'!F14)</f>
+        <f>AVERAGE(r0!F14,'r1'!F14, 'r2'!F14, 'r3'!F14)</f>
         <v>1</v>
       </c>
       <c r="G14">
-        <f>AVERAGE(r0!G14,'r1'!G14, 'r2'!G14)</f>
+        <f>AVERAGE(r0!G14,'r1'!G14, 'r2'!G14, 'r3'!G14)</f>
         <v>1</v>
       </c>
       <c r="H14">
-        <f>AVERAGE(r0!H14,'r1'!H14, 'r2'!H14)</f>
+        <f>AVERAGE(r0!H14,'r1'!H14, 'r2'!H14, 'r3'!H14)</f>
         <v>1</v>
       </c>
       <c r="I14">
-        <f>AVERAGE(r0!I14,'r1'!I14, 'r2'!I14)</f>
+        <f>AVERAGE(r0!I14,'r1'!I14, 'r2'!I14, 'r3'!I14)</f>
         <v>2</v>
       </c>
     </row>
@@ -3279,35 +3854,35 @@
         <v>10</v>
       </c>
       <c r="B15">
-        <f>AVERAGE(r0!B15,'r1'!B15, 'r2'!B15)</f>
+        <f>AVERAGE(r0!B15,'r1'!B15, 'r2'!B15, 'r3'!B15)</f>
         <v>0</v>
       </c>
       <c r="C15">
-        <f>AVERAGE(r0!C15,'r1'!C15, 'r2'!C15)</f>
+        <f>AVERAGE(r0!C15,'r1'!C15, 'r2'!C15, 'r3'!C15)</f>
         <v>0</v>
       </c>
       <c r="D15">
-        <f>AVERAGE(r0!D15,'r1'!D15, 'r2'!D15)</f>
+        <f>AVERAGE(r0!D15,'r1'!D15, 'r2'!D15, 'r3'!D15)</f>
         <v>0</v>
       </c>
       <c r="E15">
-        <f>AVERAGE(r0!E15,'r1'!E15, 'r2'!E15)</f>
+        <f>AVERAGE(r0!E15,'r1'!E15, 'r2'!E15, 'r3'!E15)</f>
         <v>0</v>
       </c>
       <c r="F15">
-        <f>AVERAGE(r0!F15,'r1'!F15, 'r2'!F15)</f>
+        <f>AVERAGE(r0!F15,'r1'!F15, 'r2'!F15, 'r3'!F15)</f>
         <v>1</v>
       </c>
       <c r="G15">
-        <f>AVERAGE(r0!G15,'r1'!G15, 'r2'!G15)</f>
+        <f>AVERAGE(r0!G15,'r1'!G15, 'r2'!G15, 'r3'!G15)</f>
         <v>0</v>
       </c>
       <c r="H15">
-        <f>AVERAGE(r0!H15,'r1'!H15, 'r2'!H15)</f>
+        <f>AVERAGE(r0!H15,'r1'!H15, 'r2'!H15, 'r3'!H15)</f>
         <v>1</v>
       </c>
       <c r="I15">
-        <f>AVERAGE(r0!I15,'r1'!I15, 'r2'!I15)</f>
+        <f>AVERAGE(r0!I15,'r1'!I15, 'r2'!I15, 'r3'!I15)</f>
         <v>0</v>
       </c>
     </row>
@@ -3316,35 +3891,35 @@
         <v>11</v>
       </c>
       <c r="B16">
-        <f>AVERAGE(r0!B16,'r1'!B16, 'r2'!B16)</f>
+        <f>AVERAGE(r0!B16,'r1'!B16, 'r2'!B16, 'r3'!B16)</f>
         <v>3</v>
       </c>
       <c r="C16">
-        <f>AVERAGE(r0!C16,'r1'!C16, 'r2'!C16)</f>
+        <f>AVERAGE(r0!C16,'r1'!C16, 'r2'!C16, 'r3'!C16)</f>
         <v>1</v>
       </c>
       <c r="D16">
-        <f>AVERAGE(r0!D16,'r1'!D16, 'r2'!D16)</f>
+        <f>AVERAGE(r0!D16,'r1'!D16, 'r2'!D16, 'r3'!D16)</f>
         <v>1</v>
       </c>
       <c r="E16">
-        <f>AVERAGE(r0!E16,'r1'!E16, 'r2'!E16)</f>
+        <f>AVERAGE(r0!E16,'r1'!E16, 'r2'!E16, 'r3'!E16)</f>
         <v>1</v>
       </c>
       <c r="F16">
-        <f>AVERAGE(r0!F16,'r1'!F16, 'r2'!F16)</f>
+        <f>AVERAGE(r0!F16,'r1'!F16, 'r2'!F16, 'r3'!F16)</f>
         <v>1</v>
       </c>
       <c r="G16">
-        <f>AVERAGE(r0!G16,'r1'!G16, 'r2'!G16)</f>
+        <f>AVERAGE(r0!G16,'r1'!G16, 'r2'!G16, 'r3'!G16)</f>
         <v>1</v>
       </c>
       <c r="H16">
-        <f>AVERAGE(r0!H16,'r1'!H16, 'r2'!H16)</f>
+        <f>AVERAGE(r0!H16,'r1'!H16, 'r2'!H16, 'r3'!H16)</f>
         <v>1</v>
       </c>
       <c r="I16">
-        <f>AVERAGE(r0!I16,'r1'!I16, 'r2'!I16)</f>
+        <f>AVERAGE(r0!I16,'r1'!I16, 'r2'!I16, 'r3'!I16)</f>
         <v>2</v>
       </c>
     </row>
@@ -3353,35 +3928,35 @@
         <v>12</v>
       </c>
       <c r="B17">
-        <f>AVERAGE(r0!B17,'r1'!B17, 'r2'!B17)</f>
+        <f>AVERAGE(r0!B17,'r1'!B17, 'r2'!B17, 'r3'!B17)</f>
         <v>3</v>
       </c>
       <c r="C17">
-        <f>AVERAGE(r0!C17,'r1'!C17, 'r2'!C17)</f>
+        <f>AVERAGE(r0!C17,'r1'!C17, 'r2'!C17, 'r3'!C17)</f>
         <v>1</v>
       </c>
       <c r="D17">
-        <f>AVERAGE(r0!D17,'r1'!D17, 'r2'!D17)</f>
+        <f>AVERAGE(r0!D17,'r1'!D17, 'r2'!D17, 'r3'!D17)</f>
         <v>1</v>
       </c>
       <c r="E17">
-        <f>AVERAGE(r0!E17,'r1'!E17, 'r2'!E17)</f>
+        <f>AVERAGE(r0!E17,'r1'!E17, 'r2'!E17, 'r3'!E17)</f>
         <v>1</v>
       </c>
       <c r="F17">
-        <f>AVERAGE(r0!F17,'r1'!F17, 'r2'!F17)</f>
+        <f>AVERAGE(r0!F17,'r1'!F17, 'r2'!F17, 'r3'!F17)</f>
         <v>1</v>
       </c>
       <c r="G17">
-        <f>AVERAGE(r0!G17,'r1'!G17, 'r2'!G17)</f>
+        <f>AVERAGE(r0!G17,'r1'!G17, 'r2'!G17, 'r3'!G17)</f>
         <v>1</v>
       </c>
       <c r="H17">
-        <f>AVERAGE(r0!H17,'r1'!H17, 'r2'!H17)</f>
+        <f>AVERAGE(r0!H17,'r1'!H17, 'r2'!H17, 'r3'!H17)</f>
         <v>1</v>
       </c>
       <c r="I17">
-        <f>AVERAGE(r0!I17,'r1'!I17, 'r2'!I17)</f>
+        <f>AVERAGE(r0!I17,'r1'!I17, 'r2'!I17, 'r3'!I17)</f>
         <v>2</v>
       </c>
     </row>
@@ -3390,35 +3965,35 @@
         <v>13</v>
       </c>
       <c r="B18">
-        <f>AVERAGE(r0!B18,'r1'!B18, 'r2'!B18)</f>
-        <v>1</v>
-      </c>
-      <c r="C18" s="1">
-        <f>AVERAGE(r0!C18,'r1'!C18, 'r2'!C18)</f>
-        <v>0.66666666666666663</v>
+        <f>AVERAGE(r0!B18,'r1'!B18, 'r2'!B18, 'r3'!B18)</f>
+        <v>0.75</v>
+      </c>
+      <c r="C18">
+        <f>AVERAGE(r0!C18,'r1'!C18, 'r2'!C18, 'r3'!C18)</f>
+        <v>0.5</v>
       </c>
       <c r="D18">
-        <f>AVERAGE(r0!D18,'r1'!D18, 'r2'!D18)</f>
+        <f>AVERAGE(r0!D18,'r1'!D18, 'r2'!D18, 'r3'!D18)</f>
         <v>0</v>
       </c>
       <c r="E18">
-        <f>AVERAGE(r0!E18,'r1'!E18, 'r2'!E18)</f>
+        <f>AVERAGE(r0!E18,'r1'!E18, 'r2'!E18, 'r3'!E18)</f>
         <v>0</v>
       </c>
       <c r="F18">
-        <f>AVERAGE(r0!F18,'r1'!F18, 'r2'!F18)</f>
+        <f>AVERAGE(r0!F18,'r1'!F18, 'r2'!F18, 'r3'!F18)</f>
         <v>0</v>
       </c>
       <c r="G18">
-        <f>AVERAGE(r0!G18,'r1'!G18, 'r2'!G18)</f>
+        <f>AVERAGE(r0!G18,'r1'!G18, 'r2'!G18, 'r3'!G18)</f>
         <v>0</v>
       </c>
       <c r="H18">
-        <f>AVERAGE(r0!H18,'r1'!H18, 'r2'!H18)</f>
+        <f>AVERAGE(r0!H18,'r1'!H18, 'r2'!H18, 'r3'!H18)</f>
         <v>0</v>
       </c>
       <c r="I18">
-        <f>AVERAGE(r0!I18,'r1'!I18, 'r2'!I18)</f>
+        <f>AVERAGE(r0!I18,'r1'!I18, 'r2'!I18, 'r3'!I18)</f>
         <v>0</v>
       </c>
     </row>
@@ -3427,35 +4002,35 @@
         <v>14</v>
       </c>
       <c r="B19">
-        <f>AVERAGE(r0!B19,'r1'!B19, 'r2'!B19)</f>
+        <f>AVERAGE(r0!B19,'r1'!B19, 'r2'!B19, 'r3'!B19)</f>
         <v>0</v>
       </c>
       <c r="C19">
-        <f>AVERAGE(r0!C19,'r1'!C19, 'r2'!C19)</f>
+        <f>AVERAGE(r0!C19,'r1'!C19, 'r2'!C19, 'r3'!C19)</f>
         <v>0</v>
       </c>
       <c r="D19">
-        <f>AVERAGE(r0!D19,'r1'!D19, 'r2'!D19)</f>
+        <f>AVERAGE(r0!D19,'r1'!D19, 'r2'!D19, 'r3'!D19)</f>
         <v>0</v>
       </c>
       <c r="E19">
-        <f>AVERAGE(r0!E19,'r1'!E19, 'r2'!E19)</f>
+        <f>AVERAGE(r0!E19,'r1'!E19, 'r2'!E19, 'r3'!E19)</f>
         <v>0</v>
       </c>
       <c r="F19">
-        <f>AVERAGE(r0!F19,'r1'!F19, 'r2'!F19)</f>
+        <f>AVERAGE(r0!F19,'r1'!F19, 'r2'!F19, 'r3'!F19)</f>
         <v>0</v>
       </c>
       <c r="G19">
-        <f>AVERAGE(r0!G19,'r1'!G19, 'r2'!G19)</f>
+        <f>AVERAGE(r0!G19,'r1'!G19, 'r2'!G19, 'r3'!G19)</f>
         <v>0</v>
       </c>
       <c r="H19">
-        <f>AVERAGE(r0!H19,'r1'!H19, 'r2'!H19)</f>
+        <f>AVERAGE(r0!H19,'r1'!H19, 'r2'!H19, 'r3'!H19)</f>
         <v>0</v>
       </c>
       <c r="I19">
-        <f>AVERAGE(r0!I19,'r1'!I19, 'r2'!I19)</f>
+        <f>AVERAGE(r0!I19,'r1'!I19, 'r2'!I19, 'r3'!I19)</f>
         <v>0</v>
       </c>
     </row>
@@ -3464,109 +4039,109 @@
         <v>15</v>
       </c>
       <c r="B20">
-        <f>AVERAGE(r0!B20,'r1'!B20, 'r2'!B20)</f>
+        <f>AVERAGE(r0!B20,'r1'!B20, 'r2'!B20, 'r3'!B20)</f>
         <v>0</v>
       </c>
       <c r="C20">
-        <f>AVERAGE(r0!C20,'r1'!C20, 'r2'!C20)</f>
-        <v>0</v>
-      </c>
-      <c r="D20" s="1">
-        <f>AVERAGE(r0!D20,'r1'!D20, 'r2'!D20)</f>
-        <v>0.33333333333333331</v>
+        <f>AVERAGE(r0!C20,'r1'!C20, 'r2'!C20, 'r3'!C20)</f>
+        <v>0</v>
+      </c>
+      <c r="D20">
+        <f>AVERAGE(r0!D20,'r1'!D20, 'r2'!D20, 'r3'!D20)</f>
+        <v>0.5</v>
       </c>
       <c r="E20">
-        <f>AVERAGE(r0!E20,'r1'!E20, 'r2'!E20)</f>
-        <v>0</v>
-      </c>
-      <c r="F20" s="1">
-        <f>AVERAGE(r0!F20,'r1'!F20, 'r2'!F20)</f>
+        <f>AVERAGE(r0!E20,'r1'!E20, 'r2'!E20, 'r3'!E20)</f>
+        <v>0</v>
+      </c>
+      <c r="F20">
+        <f>AVERAGE(r0!F20,'r1'!F20, 'r2'!F20, 'r3'!F20)</f>
         <v>0.66666666666666663</v>
       </c>
-      <c r="G20" s="1">
-        <f>AVERAGE(r0!G20,'r1'!G20, 'r2'!G20)</f>
+      <c r="G20">
+        <f>AVERAGE(r0!G20,'r1'!G20, 'r2'!G20, 'r3'!G20)</f>
         <v>1.3333333333333333</v>
       </c>
       <c r="H20">
-        <f>AVERAGE(r0!H20,'r1'!H20, 'r2'!H20)</f>
+        <f>AVERAGE(r0!H20,'r1'!H20, 'r2'!H20, 'r3'!H20)</f>
         <v>0</v>
       </c>
       <c r="I20">
-        <f>AVERAGE(r0!I20,'r1'!I20, 'r2'!I20)</f>
+        <f>AVERAGE(r0!I20,'r1'!I20, 'r2'!I20, 'r3'!I20)</f>
         <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>16</v>
-      </c>
-      <c r="B21" s="1">
-        <f>AVERAGE(r0!B21,'r1'!B21, 'r2'!B21)</f>
-        <v>25.585333333333335</v>
-      </c>
-      <c r="C21" s="1">
-        <f>AVERAGE(r0!C21,'r1'!C21, 'r2'!C21)</f>
-        <v>21.831333333333333</v>
-      </c>
-      <c r="D21" s="1">
-        <f>AVERAGE(r0!D21,'r1'!D21, 'r2'!D21)</f>
-        <v>15.663666666666666</v>
-      </c>
-      <c r="E21" s="1">
-        <f>AVERAGE(r0!E21,'r1'!E21, 'r2'!E21)</f>
-        <v>17.267666666666667</v>
-      </c>
-      <c r="F21" s="1">
-        <f>AVERAGE(r0!F21,'r1'!F21, 'r2'!F21)</f>
+        <v>55</v>
+      </c>
+      <c r="B21">
+        <f>AVERAGE(r0!B21,'r1'!B21, 'r2'!B21, 'r3'!B21)</f>
+        <v>25.304000000000002</v>
+      </c>
+      <c r="C21">
+        <f>AVERAGE(r0!C21,'r1'!C21, 'r2'!C21, 'r3'!C21)</f>
+        <v>21.376249999999999</v>
+      </c>
+      <c r="D21">
+        <f>AVERAGE(r0!D21,'r1'!D21, 'r2'!D21, 'r3'!D21)</f>
+        <v>15.272</v>
+      </c>
+      <c r="E21">
+        <f>AVERAGE(r0!E21,'r1'!E21, 'r2'!E21, 'r3'!E21)</f>
+        <v>17.91075</v>
+      </c>
+      <c r="F21">
+        <f>AVERAGE(r0!F21,'r1'!F21, 'r2'!F21, 'r3'!F21)</f>
         <v>12.766666666666666</v>
       </c>
-      <c r="G21" s="1">
-        <f>AVERAGE(r0!G21,'r1'!G21, 'r2'!G21)</f>
+      <c r="G21">
+        <f>AVERAGE(r0!G21,'r1'!G21, 'r2'!G21, 'r3'!G21)</f>
         <v>13.334333333333333</v>
       </c>
-      <c r="H21" s="1">
-        <f>AVERAGE(r0!H21,'r1'!H21, 'r2'!H21)</f>
+      <c r="H21">
+        <f>AVERAGE(r0!H21,'r1'!H21, 'r2'!H21, 'r3'!H21)</f>
         <v>17.989000000000001</v>
       </c>
-      <c r="I21" s="1">
-        <f>AVERAGE(r0!I21,'r1'!I21, 'r2'!I21)</f>
+      <c r="I21">
+        <f>AVERAGE(r0!I21,'r1'!I21, 'r2'!I21, 'r3'!I21)</f>
         <v>15.735666666666667</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>19</v>
-      </c>
-      <c r="B22" s="1">
-        <f>AVERAGE(r0!B22,'r1'!B22, 'r2'!B22)</f>
-        <v>2.4386666666666668E-2</v>
-      </c>
-      <c r="C22" s="1">
-        <f>AVERAGE(r0!C22,'r1'!C22, 'r2'!C22)</f>
-        <v>2.2651000000000001E-2</v>
-      </c>
-      <c r="D22" s="1">
-        <f>AVERAGE(r0!D22,'r1'!D22, 'r2'!D22)</f>
-        <v>1.8483666666666666E-2</v>
-      </c>
-      <c r="E22" s="1">
-        <f>AVERAGE(r0!E22,'r1'!E22, 'r2'!E22)</f>
-        <v>2.0503E-2</v>
-      </c>
-      <c r="F22" s="1">
-        <f>AVERAGE(r0!F22,'r1'!F22, 'r2'!F22)</f>
+        <v>54</v>
+      </c>
+      <c r="B22">
+        <f>AVERAGE(r0!B22,'r1'!B22, 'r2'!B22, 'r3'!B22)</f>
+        <v>2.4203500000000003E-2</v>
+      </c>
+      <c r="C22">
+        <f>AVERAGE(r0!C22,'r1'!C22, 'r2'!C22, 'r3'!C22)</f>
+        <v>2.2918250000000001E-2</v>
+      </c>
+      <c r="D22">
+        <f>AVERAGE(r0!D22,'r1'!D22, 'r2'!D22, 'r3'!D22)</f>
+        <v>1.7138500000000001E-2</v>
+      </c>
+      <c r="E22">
+        <f>AVERAGE(r0!E22,'r1'!E22, 'r2'!E22, 'r3'!E22)</f>
+        <v>1.9991000000000002E-2</v>
+      </c>
+      <c r="F22">
+        <f>AVERAGE(r0!F22,'r1'!F22, 'r2'!F22, 'r3'!F22)</f>
         <v>1.6129333333333332E-2</v>
       </c>
-      <c r="G22" s="1">
-        <f>AVERAGE(r0!G22,'r1'!G22, 'r2'!G22)</f>
+      <c r="G22">
+        <f>AVERAGE(r0!G22,'r1'!G22, 'r2'!G22, 'r3'!G22)</f>
         <v>1.4313666666666664E-2</v>
       </c>
-      <c r="H22" s="1">
-        <f>AVERAGE(r0!H22,'r1'!H22, 'r2'!H22)</f>
+      <c r="H22">
+        <f>AVERAGE(r0!H22,'r1'!H22, 'r2'!H22, 'r3'!H22)</f>
         <v>1.5993333333333335E-2</v>
       </c>
-      <c r="I22" s="1">
-        <f>AVERAGE(r0!I22,'r1'!I22, 'r2'!I22)</f>
+      <c r="I22">
+        <f>AVERAGE(r0!I22,'r1'!I22, 'r2'!I22, 'r3'!I22)</f>
         <v>1.7988666666666667E-2</v>
       </c>
     </row>
@@ -3584,7 +4159,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE3232CA-EC8E-404A-B90B-03381B7790AE}">
   <dimension ref="A1:I23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
added r4 results data
</commit_message>
<xml_diff>
--- a/finalReport.xlsx
+++ b/finalReport.xlsx
@@ -8,17 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fedev\Documents\UNICAM\Phd\unmock\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB7B02E2-6D69-4B19-A4B0-41F710271219}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50CE2DFE-0E9C-489B-B7E8-2C990D3099A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{A0F7C0B4-A897-4B1D-9E87-712A814F4D93}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{A0F7C0B4-A897-4B1D-9E87-712A814F4D93}"/>
   </bookViews>
   <sheets>
     <sheet name="r0" sheetId="1" r:id="rId1"/>
     <sheet name="r1" sheetId="2" r:id="rId2"/>
     <sheet name="r2" sheetId="5" r:id="rId3"/>
     <sheet name="r3" sheetId="6" r:id="rId4"/>
-    <sheet name="global" sheetId="4" r:id="rId5"/>
-    <sheet name="Test IDs" sheetId="3" r:id="rId6"/>
+    <sheet name="r4" sheetId="7" r:id="rId5"/>
+    <sheet name="global" sheetId="4" r:id="rId6"/>
+    <sheet name="Test IDs" sheetId="3" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="56">
   <si>
     <t>Target test</t>
   </si>
@@ -262,12 +263,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -2250,7 +2252,7 @@
         <v>1</v>
       </c>
       <c r="H7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I7">
         <v>1</v>
@@ -2279,7 +2281,7 @@
         <v>1</v>
       </c>
       <c r="H8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I8">
         <v>0</v>
@@ -2308,7 +2310,7 @@
         <v>0</v>
       </c>
       <c r="H9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I9">
         <v>0</v>
@@ -3232,7 +3234,7 @@
         <v>1</v>
       </c>
       <c r="I16">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
@@ -3261,7 +3263,7 @@
         <v>1</v>
       </c>
       <c r="I17">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
@@ -3473,6 +3475,724 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF8B6B79-B979-4750-9A5D-E8DD6E5A0363}">
+  <dimension ref="A1:I24"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="55.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="9" width="11.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="str">
+        <f>'Test IDs'!C2</f>
+        <v>DS.1</v>
+      </c>
+      <c r="C1" t="str">
+        <f>'Test IDs'!C3</f>
+        <v>DS.2</v>
+      </c>
+      <c r="D1" t="str">
+        <f>'Test IDs'!C4</f>
+        <v>DS.3</v>
+      </c>
+      <c r="E1" t="str">
+        <f>'Test IDs'!C5</f>
+        <v>DS.4</v>
+      </c>
+      <c r="F1" t="str">
+        <f>'Test IDs'!C6</f>
+        <v>N.1</v>
+      </c>
+      <c r="G1" t="str">
+        <f>'Test IDs'!C7</f>
+        <v>N.2</v>
+      </c>
+      <c r="H1" t="str">
+        <f>'Test IDs'!C8</f>
+        <v>N.3</v>
+      </c>
+      <c r="I1" t="str">
+        <f>'Test IDs'!C9</f>
+        <v>N.4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>3</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6">
+        <v>1</v>
+      </c>
+      <c r="I6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>0</v>
+      </c>
+      <c r="C7">
+        <v>2</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="G7">
+        <v>1</v>
+      </c>
+      <c r="H7">
+        <v>1</v>
+      </c>
+      <c r="I7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>0</v>
+      </c>
+      <c r="C8">
+        <v>0</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <v>0</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8">
+        <v>0</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>0</v>
+      </c>
+      <c r="C9">
+        <v>0</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="F9">
+        <v>0</v>
+      </c>
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9">
+        <v>0</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>50</v>
+      </c>
+      <c r="B10">
+        <v>0</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <v>0</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <v>0</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>51</v>
+      </c>
+      <c r="B11">
+        <v>0</v>
+      </c>
+      <c r="C11">
+        <v>1</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11">
+        <v>0</v>
+      </c>
+      <c r="F11">
+        <v>0</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11">
+        <v>0</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>52</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12">
+        <v>0</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="F12">
+        <v>0</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="I12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>53</v>
+      </c>
+      <c r="B13">
+        <v>0</v>
+      </c>
+      <c r="C13">
+        <v>0</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+      <c r="F13">
+        <v>0</v>
+      </c>
+      <c r="G13">
+        <v>0</v>
+      </c>
+      <c r="H13">
+        <v>0</v>
+      </c>
+      <c r="I13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>9</v>
+      </c>
+      <c r="B14">
+        <v>3</v>
+      </c>
+      <c r="C14">
+        <v>1</v>
+      </c>
+      <c r="D14">
+        <v>1</v>
+      </c>
+      <c r="E14">
+        <v>1</v>
+      </c>
+      <c r="F14">
+        <v>1</v>
+      </c>
+      <c r="G14">
+        <v>1</v>
+      </c>
+      <c r="H14">
+        <v>1</v>
+      </c>
+      <c r="I14">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>10</v>
+      </c>
+      <c r="B15">
+        <v>0</v>
+      </c>
+      <c r="C15">
+        <v>0</v>
+      </c>
+      <c r="D15">
+        <v>0</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+      <c r="F15">
+        <v>1</v>
+      </c>
+      <c r="G15">
+        <v>0</v>
+      </c>
+      <c r="H15">
+        <v>1</v>
+      </c>
+      <c r="I15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>11</v>
+      </c>
+      <c r="B16">
+        <v>3</v>
+      </c>
+      <c r="C16">
+        <v>1</v>
+      </c>
+      <c r="D16">
+        <v>1</v>
+      </c>
+      <c r="E16">
+        <v>1</v>
+      </c>
+      <c r="F16">
+        <v>1</v>
+      </c>
+      <c r="G16">
+        <v>1</v>
+      </c>
+      <c r="H16">
+        <v>1</v>
+      </c>
+      <c r="I16">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>12</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17">
+        <v>1</v>
+      </c>
+      <c r="D17">
+        <v>1</v>
+      </c>
+      <c r="E17">
+        <v>1</v>
+      </c>
+      <c r="F17">
+        <v>1</v>
+      </c>
+      <c r="G17">
+        <v>1</v>
+      </c>
+      <c r="H17">
+        <v>1</v>
+      </c>
+      <c r="I17">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>13</v>
+      </c>
+      <c r="B18">
+        <v>0</v>
+      </c>
+      <c r="C18">
+        <v>0</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18">
+        <v>0</v>
+      </c>
+      <c r="F18">
+        <v>0</v>
+      </c>
+      <c r="G18">
+        <v>0</v>
+      </c>
+      <c r="H18">
+        <v>0</v>
+      </c>
+      <c r="I18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>14</v>
+      </c>
+      <c r="B19">
+        <v>0</v>
+      </c>
+      <c r="C19">
+        <v>0</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19">
+        <v>0</v>
+      </c>
+      <c r="F19">
+        <v>0</v>
+      </c>
+      <c r="G19">
+        <v>0</v>
+      </c>
+      <c r="H19">
+        <v>0</v>
+      </c>
+      <c r="I19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>15</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20">
+        <v>0</v>
+      </c>
+      <c r="D20">
+        <v>0</v>
+      </c>
+      <c r="E20">
+        <v>0</v>
+      </c>
+      <c r="F20">
+        <v>1</v>
+      </c>
+      <c r="G20">
+        <v>0</v>
+      </c>
+      <c r="H20">
+        <v>0</v>
+      </c>
+      <c r="I20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>16</v>
+      </c>
+      <c r="B21" s="1">
+        <v>22.710999999999999</v>
+      </c>
+      <c r="C21" s="1">
+        <v>19.094999999999999</v>
+      </c>
+      <c r="D21" s="1">
+        <v>12.407999999999999</v>
+      </c>
+      <c r="E21" s="1">
+        <v>15.888999999999999</v>
+      </c>
+      <c r="F21" s="1">
+        <v>13.079000000000001</v>
+      </c>
+      <c r="G21" s="1">
+        <v>7.7080000000000002</v>
+      </c>
+      <c r="H21" s="1">
+        <v>11.324999999999999</v>
+      </c>
+      <c r="I21" s="1">
+        <v>13.55</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>19</v>
+      </c>
+      <c r="B22" s="1">
+        <v>2.4306999999999999E-2</v>
+      </c>
+      <c r="C22" s="1">
+        <v>2.0389000000000001E-2</v>
+      </c>
+      <c r="D22" s="1">
+        <v>1.2661E-2</v>
+      </c>
+      <c r="E22" s="1">
+        <v>1.8346999999999999E-2</v>
+      </c>
+      <c r="F22" s="1">
+        <v>1.3339E-2</v>
+      </c>
+      <c r="G22" s="1">
+        <v>9.0679999999999997E-3</v>
+      </c>
+      <c r="H22" s="1">
+        <v>1.2078999999999999E-2</v>
+      </c>
+      <c r="I22" s="1">
+        <v>1.4545000000000001E-2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>17</v>
+      </c>
+      <c r="B23" t="s">
+        <v>18</v>
+      </c>
+      <c r="C23" t="s">
+        <v>18</v>
+      </c>
+      <c r="D23" t="s">
+        <v>18</v>
+      </c>
+      <c r="E23" t="s">
+        <v>18</v>
+      </c>
+      <c r="F23" t="s">
+        <v>18</v>
+      </c>
+      <c r="G23" t="s">
+        <v>18</v>
+      </c>
+      <c r="H23" t="s">
+        <v>18</v>
+      </c>
+      <c r="I23" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>20</v>
+      </c>
+      <c r="B24" t="s">
+        <v>21</v>
+      </c>
+      <c r="C24" t="s">
+        <v>21</v>
+      </c>
+      <c r="D24" t="s">
+        <v>21</v>
+      </c>
+      <c r="E24" t="s">
+        <v>21</v>
+      </c>
+      <c r="F24" t="s">
+        <v>22</v>
+      </c>
+      <c r="G24" t="s">
+        <v>21</v>
+      </c>
+      <c r="H24" t="s">
+        <v>22</v>
+      </c>
+      <c r="I24" t="s">
+        <v>22</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E040BF79-8B7D-43C4-816A-164CB83CAB3E}">
   <dimension ref="A1:I23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3524,35 +4244,35 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <f>AVERAGE(r0!B2,'r1'!B2, 'r2'!B2, 'r3'!B2)</f>
+        <f>AVERAGE(r0!B2,'r1'!B2, 'r2'!B2, 'r3'!B2, 'r4'!B2)</f>
         <v>3</v>
       </c>
       <c r="C2">
-        <f>AVERAGE(r0!C2,'r1'!C2, 'r2'!C2, 'r3'!C2)</f>
+        <f>AVERAGE(r0!C2,'r1'!C2, 'r2'!C2, 'r3'!C2, 'r4'!C2)</f>
         <v>2</v>
       </c>
       <c r="D2">
-        <f>AVERAGE(r0!D2,'r1'!D2, 'r2'!D2, 'r3'!D2)</f>
+        <f>AVERAGE(r0!D2,'r1'!D2, 'r2'!D2, 'r3'!D2, 'r4'!D2)</f>
         <v>1</v>
       </c>
       <c r="E2">
-        <f>AVERAGE(r0!E2,'r1'!E2, 'r2'!E2, 'r3'!E2)</f>
+        <f>AVERAGE(r0!E2,'r1'!E2, 'r2'!E2, 'r3'!E2, 'r4'!E2)</f>
         <v>1</v>
       </c>
       <c r="F2">
-        <f>AVERAGE(r0!F2,'r1'!F2, 'r2'!F2, 'r3'!F2)</f>
+        <f>AVERAGE(r0!F2,'r1'!F2, 'r2'!F2, 'r3'!F2, 'r4'!F2)</f>
         <v>1</v>
       </c>
       <c r="G2">
-        <f>AVERAGE(r0!G2,'r1'!G2, 'r2'!G2, 'r3'!G2)</f>
+        <f>AVERAGE(r0!G2,'r1'!G2, 'r2'!G2, 'r3'!G2, 'r4'!G2)</f>
         <v>0</v>
       </c>
       <c r="H2">
-        <f>AVERAGE(r0!H2,'r1'!H2, 'r2'!H2, 'r3'!H2)</f>
+        <f>AVERAGE(r0!H2,'r1'!H2, 'r2'!H2, 'r3'!H2, 'r4'!H2)</f>
         <v>0</v>
       </c>
       <c r="I2">
-        <f>AVERAGE(r0!I2,'r1'!I2, 'r2'!I2, 'r3'!I2)</f>
+        <f>AVERAGE(r0!I2,'r1'!I2, 'r2'!I2, 'r3'!I2, 'r4'!I2)</f>
         <v>1</v>
       </c>
     </row>
@@ -3561,35 +4281,35 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <f>AVERAGE(r0!B3,'r1'!B3, 'r2'!B3, 'r3'!B3)</f>
+        <f>AVERAGE(r0!B3,'r1'!B3, 'r2'!B3, 'r3'!B3, 'r4'!B3)</f>
         <v>3</v>
       </c>
       <c r="C3">
-        <f>AVERAGE(r0!C3,'r1'!C3, 'r2'!C3, 'r3'!C3)</f>
+        <f>AVERAGE(r0!C3,'r1'!C3, 'r2'!C3, 'r3'!C3, 'r4'!C3)</f>
         <v>2</v>
       </c>
       <c r="D3">
-        <f>AVERAGE(r0!D3,'r1'!D3, 'r2'!D3, 'r3'!D3)</f>
+        <f>AVERAGE(r0!D3,'r1'!D3, 'r2'!D3, 'r3'!D3, 'r4'!D3)</f>
         <v>1</v>
       </c>
       <c r="E3">
-        <f>AVERAGE(r0!E3,'r1'!E3, 'r2'!E3, 'r3'!E3)</f>
+        <f>AVERAGE(r0!E3,'r1'!E3, 'r2'!E3, 'r3'!E3, 'r4'!E3)</f>
         <v>1</v>
       </c>
       <c r="F3">
-        <f>AVERAGE(r0!F3,'r1'!F3, 'r2'!F3, 'r3'!F3)</f>
+        <f>AVERAGE(r0!F3,'r1'!F3, 'r2'!F3, 'r3'!F3, 'r4'!F3)</f>
         <v>1</v>
       </c>
       <c r="G3">
-        <f>AVERAGE(r0!G3,'r1'!G3, 'r2'!G3, 'r3'!G3)</f>
+        <f>AVERAGE(r0!G3,'r1'!G3, 'r2'!G3, 'r3'!G3, 'r4'!G3)</f>
         <v>0</v>
       </c>
       <c r="H3">
-        <f>AVERAGE(r0!H3,'r1'!H3, 'r2'!H3, 'r3'!H3)</f>
+        <f>AVERAGE(r0!H3,'r1'!H3, 'r2'!H3, 'r3'!H3, 'r4'!H3)</f>
         <v>0</v>
       </c>
       <c r="I3">
-        <f>AVERAGE(r0!I3,'r1'!I3, 'r2'!I3, 'r3'!I3)</f>
+        <f>AVERAGE(r0!I3,'r1'!I3, 'r2'!I3, 'r3'!I3, 'r4'!I3)</f>
         <v>1</v>
       </c>
     </row>
@@ -3598,35 +4318,35 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <f>AVERAGE(r0!B4,'r1'!B4, 'r2'!B4, 'r3'!B4)</f>
+        <f>AVERAGE(r0!B4,'r1'!B4, 'r2'!B4, 'r3'!B4, 'r4'!B4)</f>
         <v>0</v>
       </c>
       <c r="C4">
-        <f>AVERAGE(r0!C4,'r1'!C4, 'r2'!C4, 'r3'!C4)</f>
+        <f>AVERAGE(r0!C4,'r1'!C4, 'r2'!C4, 'r3'!C4, 'r4'!C4)</f>
         <v>0</v>
       </c>
       <c r="D4">
-        <f>AVERAGE(r0!D4,'r1'!D4, 'r2'!D4, 'r3'!D4)</f>
+        <f>AVERAGE(r0!D4,'r1'!D4, 'r2'!D4, 'r3'!D4, 'r4'!D4)</f>
         <v>0</v>
       </c>
       <c r="E4">
-        <f>AVERAGE(r0!E4,'r1'!E4, 'r2'!E4, 'r3'!E4)</f>
+        <f>AVERAGE(r0!E4,'r1'!E4, 'r2'!E4, 'r3'!E4, 'r4'!E4)</f>
         <v>0</v>
       </c>
       <c r="F4">
-        <f>AVERAGE(r0!F4,'r1'!F4, 'r2'!F4, 'r3'!F4)</f>
+        <f>AVERAGE(r0!F4,'r1'!F4, 'r2'!F4, 'r3'!F4, 'r4'!F4)</f>
         <v>0</v>
       </c>
       <c r="G4">
-        <f>AVERAGE(r0!G4,'r1'!G4, 'r2'!G4, 'r3'!G4)</f>
+        <f>AVERAGE(r0!G4,'r1'!G4, 'r2'!G4, 'r3'!G4, 'r4'!G4)</f>
         <v>0</v>
       </c>
       <c r="H4">
-        <f>AVERAGE(r0!H4,'r1'!H4, 'r2'!H4, 'r3'!H4)</f>
+        <f>AVERAGE(r0!H4,'r1'!H4, 'r2'!H4, 'r3'!H4, 'r4'!H4)</f>
         <v>0</v>
       </c>
       <c r="I4">
-        <f>AVERAGE(r0!I4,'r1'!I4, 'r2'!I4, 'r3'!I4)</f>
+        <f>AVERAGE(r0!I4,'r1'!I4, 'r2'!I4, 'r3'!I4, 'r4'!I4)</f>
         <v>0</v>
       </c>
     </row>
@@ -3635,35 +4355,35 @@
         <v>4</v>
       </c>
       <c r="B5" s="1">
-        <f>AVERAGE(r0!B5,'r1'!B5, 'r2'!B5, 'r3'!B5)</f>
-        <v>0.75</v>
+        <f>AVERAGE(r0!B5,'r1'!B5, 'r2'!B5, 'r3'!B5, 'r4'!B5)</f>
+        <v>0.6</v>
       </c>
       <c r="C5" s="1">
-        <f>AVERAGE(r0!C5,'r1'!C5, 'r2'!C5, 'r3'!C5)</f>
-        <v>0.25</v>
+        <f>AVERAGE(r0!C5,'r1'!C5, 'r2'!C5, 'r3'!C5, 'r4'!C5)</f>
+        <v>0.2</v>
       </c>
       <c r="D5">
-        <f>AVERAGE(r0!D5,'r1'!D5, 'r2'!D5, 'r3'!D5)</f>
+        <f>AVERAGE(r0!D5,'r1'!D5, 'r2'!D5, 'r3'!D5, 'r4'!D5)</f>
         <v>0</v>
       </c>
       <c r="E5">
-        <f>AVERAGE(r0!E5,'r1'!E5, 'r2'!E5, 'r3'!E5)</f>
+        <f>AVERAGE(r0!E5,'r1'!E5, 'r2'!E5, 'r3'!E5, 'r4'!E5)</f>
         <v>0</v>
       </c>
       <c r="F5">
-        <f>AVERAGE(r0!F5,'r1'!F5, 'r2'!F5, 'r3'!F5)</f>
+        <f>AVERAGE(r0!F5,'r1'!F5, 'r2'!F5, 'r3'!F5, 'r4'!F5)</f>
         <v>0</v>
       </c>
       <c r="G5">
-        <f>AVERAGE(r0!G5,'r1'!G5, 'r2'!G5, 'r3'!G5)</f>
+        <f>AVERAGE(r0!G5,'r1'!G5, 'r2'!G5, 'r3'!G5, 'r4'!G5)</f>
         <v>0</v>
       </c>
       <c r="H5">
-        <f>AVERAGE(r0!H5,'r1'!H5, 'r2'!H5, 'r3'!H5)</f>
+        <f>AVERAGE(r0!H5,'r1'!H5, 'r2'!H5, 'r3'!H5, 'r4'!H5)</f>
         <v>0</v>
       </c>
       <c r="I5">
-        <f>AVERAGE(r0!I5,'r1'!I5, 'r2'!I5, 'r3'!I5)</f>
+        <f>AVERAGE(r0!I5,'r1'!I5, 'r2'!I5, 'r3'!I5, 'r4'!I5)</f>
         <v>0</v>
       </c>
     </row>
@@ -3672,35 +4392,35 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <f>AVERAGE(r0!B6,'r1'!B6, 'r2'!B6, 'r3'!B6)</f>
+        <f>AVERAGE(r0!B6,'r1'!B6, 'r2'!B6, 'r3'!B6, 'r4'!B6)</f>
         <v>0</v>
       </c>
       <c r="C6">
-        <f>AVERAGE(r0!C6,'r1'!C6, 'r2'!C6, 'r3'!C6)</f>
+        <f>AVERAGE(r0!C6,'r1'!C6, 'r2'!C6, 'r3'!C6, 'r4'!C6)</f>
         <v>2</v>
       </c>
       <c r="D6">
-        <f>AVERAGE(r0!D6,'r1'!D6, 'r2'!D6, 'r3'!D6)</f>
+        <f>AVERAGE(r0!D6,'r1'!D6, 'r2'!D6, 'r3'!D6, 'r4'!D6)</f>
         <v>0</v>
       </c>
       <c r="E6">
-        <f>AVERAGE(r0!E6,'r1'!E6, 'r2'!E6, 'r3'!E6)</f>
+        <f>AVERAGE(r0!E6,'r1'!E6, 'r2'!E6, 'r3'!E6, 'r4'!E6)</f>
         <v>0</v>
       </c>
       <c r="F6">
-        <f>AVERAGE(r0!F6,'r1'!F6, 'r2'!F6, 'r3'!F6)</f>
+        <f>AVERAGE(r0!F6,'r1'!F6, 'r2'!F6, 'r3'!F6, 'r4'!F6)</f>
         <v>0</v>
       </c>
       <c r="G6">
-        <f>AVERAGE(r0!G6,'r1'!G6, 'r2'!G6, 'r3'!G6)</f>
+        <f>AVERAGE(r0!G6,'r1'!G6, 'r2'!G6, 'r3'!G6, 'r4'!G6)</f>
         <v>1</v>
       </c>
       <c r="H6">
-        <f>AVERAGE(r0!H6,'r1'!H6, 'r2'!H6, 'r3'!H6)</f>
+        <f>AVERAGE(r0!H6,'r1'!H6, 'r2'!H6, 'r3'!H6, 'r4'!H6)</f>
         <v>1</v>
       </c>
       <c r="I6">
-        <f>AVERAGE(r0!I6,'r1'!I6, 'r2'!I6, 'r3'!I6)</f>
+        <f>AVERAGE(r0!I6,'r1'!I6, 'r2'!I6, 'r3'!I6, 'r4'!I6)</f>
         <v>1</v>
       </c>
     </row>
@@ -3709,35 +4429,35 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <f>AVERAGE(r0!B7,'r1'!B7, 'r2'!B7, 'r3'!B7)</f>
+        <f>AVERAGE(r0!B7,'r1'!B7, 'r2'!B7, 'r3'!B7, 'r4'!B7)</f>
         <v>0</v>
       </c>
       <c r="C7">
-        <f>AVERAGE(r0!C7,'r1'!C7, 'r2'!C7, 'r3'!C7)</f>
+        <f>AVERAGE(r0!C7,'r1'!C7, 'r2'!C7, 'r3'!C7, 'r4'!C7)</f>
         <v>2</v>
       </c>
       <c r="D7">
-        <f>AVERAGE(r0!D7,'r1'!D7, 'r2'!D7, 'r3'!D7)</f>
+        <f>AVERAGE(r0!D7,'r1'!D7, 'r2'!D7, 'r3'!D7, 'r4'!D7)</f>
         <v>0</v>
       </c>
       <c r="E7">
-        <f>AVERAGE(r0!E7,'r1'!E7, 'r2'!E7, 'r3'!E7)</f>
+        <f>AVERAGE(r0!E7,'r1'!E7, 'r2'!E7, 'r3'!E7, 'r4'!E7)</f>
         <v>0</v>
       </c>
       <c r="F7">
-        <f>AVERAGE(r0!F7,'r1'!F7, 'r2'!F7, 'r3'!F7)</f>
+        <f>AVERAGE(r0!F7,'r1'!F7, 'r2'!F7, 'r3'!F7, 'r4'!F7)</f>
         <v>0</v>
       </c>
       <c r="G7">
-        <f>AVERAGE(r0!G7,'r1'!G7, 'r2'!G7, 'r3'!G7)</f>
-        <v>1</v>
-      </c>
-      <c r="H7" s="1">
-        <f>AVERAGE(r0!H7,'r1'!H7, 'r2'!H7, 'r3'!H7)</f>
-        <v>0.75</v>
+        <f>AVERAGE(r0!G7,'r1'!G7, 'r2'!G7, 'r3'!G7, 'r4'!G7)</f>
+        <v>1</v>
+      </c>
+      <c r="H7" s="5">
+        <f>AVERAGE(r0!H7,'r1'!H7, 'r2'!H7, 'r3'!H7, 'r4'!H7)</f>
+        <v>1</v>
       </c>
       <c r="I7">
-        <f>AVERAGE(r0!I7,'r1'!I7, 'r2'!I7, 'r3'!I7)</f>
+        <f>AVERAGE(r0!I7,'r1'!I7, 'r2'!I7, 'r3'!I7, 'r4'!I7)</f>
         <v>1</v>
       </c>
     </row>
@@ -3746,35 +4466,35 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <f>AVERAGE(r0!B8,'r1'!B8, 'r2'!B8, 'r3'!B8)</f>
+        <f>AVERAGE(r0!B8,'r1'!B8, 'r2'!B8, 'r3'!B8, 'r4'!B8)</f>
         <v>0</v>
       </c>
       <c r="C8">
-        <f>AVERAGE(r0!C8,'r1'!C8, 'r2'!C8, 'r3'!C8)</f>
+        <f>AVERAGE(r0!C8,'r1'!C8, 'r2'!C8, 'r3'!C8, 'r4'!C8)</f>
         <v>0</v>
       </c>
       <c r="D8">
-        <f>AVERAGE(r0!D8,'r1'!D8, 'r2'!D8, 'r3'!D8)</f>
+        <f>AVERAGE(r0!D8,'r1'!D8, 'r2'!D8, 'r3'!D8, 'r4'!D8)</f>
         <v>0</v>
       </c>
       <c r="E8">
-        <f>AVERAGE(r0!E8,'r1'!E8, 'r2'!E8, 'r3'!E8)</f>
+        <f>AVERAGE(r0!E8,'r1'!E8, 'r2'!E8, 'r3'!E8, 'r4'!E8)</f>
         <v>0</v>
       </c>
       <c r="F8">
-        <f>AVERAGE(r0!F8,'r1'!F8, 'r2'!F8, 'r3'!F8)</f>
+        <f>AVERAGE(r0!F8,'r1'!F8, 'r2'!F8, 'r3'!F8, 'r4'!F8)</f>
         <v>0</v>
       </c>
       <c r="G8" s="1">
-        <f>AVERAGE(r0!G8,'r1'!G8, 'r2'!G8, 'r3'!G8)</f>
-        <v>0.25</v>
-      </c>
-      <c r="H8" s="1">
-        <f>AVERAGE(r0!H8,'r1'!H8, 'r2'!H8, 'r3'!H8)</f>
-        <v>0.25</v>
+        <f>AVERAGE(r0!G8,'r1'!G8, 'r2'!G8, 'r3'!G8, 'r4'!G8)</f>
+        <v>0.2</v>
+      </c>
+      <c r="H8" s="5">
+        <f>AVERAGE(r0!H8,'r1'!H8, 'r2'!H8, 'r3'!H8, 'r4'!H8)</f>
+        <v>0</v>
       </c>
       <c r="I8">
-        <f>AVERAGE(r0!I8,'r1'!I8, 'r2'!I8, 'r3'!I8)</f>
+        <f>AVERAGE(r0!I8,'r1'!I8, 'r2'!I8, 'r3'!I8, 'r4'!I8)</f>
         <v>0</v>
       </c>
     </row>
@@ -3783,35 +4503,35 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <f>AVERAGE(r0!B9,'r1'!B9, 'r2'!B9, 'r3'!B9)</f>
+        <f>AVERAGE(r0!B9,'r1'!B9, 'r2'!B9, 'r3'!B9, 'r4'!B9)</f>
         <v>0</v>
       </c>
       <c r="C9">
-        <f>AVERAGE(r0!C9,'r1'!C9, 'r2'!C9, 'r3'!C9)</f>
+        <f>AVERAGE(r0!C9,'r1'!C9, 'r2'!C9, 'r3'!C9, 'r4'!C9)</f>
         <v>0</v>
       </c>
       <c r="D9">
-        <f>AVERAGE(r0!D9,'r1'!D9, 'r2'!D9, 'r3'!D9)</f>
+        <f>AVERAGE(r0!D9,'r1'!D9, 'r2'!D9, 'r3'!D9, 'r4'!D9)</f>
         <v>0</v>
       </c>
       <c r="E9">
-        <f>AVERAGE(r0!E9,'r1'!E9, 'r2'!E9, 'r3'!E9)</f>
+        <f>AVERAGE(r0!E9,'r1'!E9, 'r2'!E9, 'r3'!E9, 'r4'!E9)</f>
         <v>0</v>
       </c>
       <c r="F9">
-        <f>AVERAGE(r0!F9,'r1'!F9, 'r2'!F9, 'r3'!F9)</f>
+        <f>AVERAGE(r0!F9,'r1'!F9, 'r2'!F9, 'r3'!F9, 'r4'!F9)</f>
         <v>0</v>
       </c>
       <c r="G9">
-        <f>AVERAGE(r0!G9,'r1'!G9, 'r2'!G9, 'r3'!G9)</f>
+        <f>AVERAGE(r0!G9,'r1'!G9, 'r2'!G9, 'r3'!G9, 'r4'!G9)</f>
         <v>0</v>
       </c>
       <c r="H9" s="1">
-        <f>AVERAGE(r0!H9,'r1'!H9, 'r2'!H9, 'r3'!H9)</f>
-        <v>0.25</v>
+        <f>AVERAGE(r0!H9,'r1'!H9, 'r2'!H9, 'r3'!H9, 'r4'!H9)</f>
+        <v>0.4</v>
       </c>
       <c r="I9">
-        <f>AVERAGE(r0!I9,'r1'!I9, 'r2'!I9, 'r3'!I9)</f>
+        <f>AVERAGE(r0!I9,'r1'!I9, 'r2'!I9, 'r3'!I9, 'r4'!I9)</f>
         <v>0</v>
       </c>
     </row>
@@ -3820,35 +4540,35 @@
         <v>50</v>
       </c>
       <c r="B10">
-        <f>AVERAGE(r0!B10,'r1'!B10, 'r2'!B10, 'r3'!B10)</f>
+        <f>AVERAGE(r0!B10,'r1'!B10, 'r2'!B10, 'r3'!B10, 'r4'!B10)</f>
         <v>0</v>
       </c>
       <c r="C10">
-        <f>AVERAGE(r0!C10,'r1'!C10, 'r2'!C10, 'r3'!C10)</f>
+        <f>AVERAGE(r0!C10,'r1'!C10, 'r2'!C10, 'r3'!C10, 'r4'!C10)</f>
         <v>1</v>
       </c>
       <c r="D10">
-        <f>AVERAGE(r0!D10,'r1'!D10, 'r2'!D10, 'r3'!D10)</f>
+        <f>AVERAGE(r0!D10,'r1'!D10, 'r2'!D10, 'r3'!D10, 'r4'!D10)</f>
         <v>0</v>
       </c>
       <c r="E10">
-        <f>AVERAGE(r0!E10,'r1'!E10, 'r2'!E10, 'r3'!E10)</f>
+        <f>AVERAGE(r0!E10,'r1'!E10, 'r2'!E10, 'r3'!E10, 'r4'!E10)</f>
         <v>0</v>
       </c>
       <c r="F10">
-        <f>AVERAGE(r0!F10,'r1'!F10, 'r2'!F10, 'r3'!F10)</f>
+        <f>AVERAGE(r0!F10,'r1'!F10, 'r2'!F10, 'r3'!F10, 'r4'!F10)</f>
         <v>0</v>
       </c>
       <c r="G10">
-        <f>AVERAGE(r0!G10,'r1'!G10, 'r2'!G10, 'r3'!G10)</f>
+        <f>AVERAGE(r0!G10,'r1'!G10, 'r2'!G10, 'r3'!G10, 'r4'!G10)</f>
         <v>0</v>
       </c>
       <c r="H10">
-        <f>AVERAGE(r0!H10,'r1'!H10, 'r2'!H10, 'r3'!H10)</f>
+        <f>AVERAGE(r0!H10,'r1'!H10, 'r2'!H10, 'r3'!H10, 'r4'!H10)</f>
         <v>0</v>
       </c>
       <c r="I10">
-        <f>AVERAGE(r0!I10,'r1'!I10, 'r2'!I10, 'r3'!I10)</f>
+        <f>AVERAGE(r0!I10,'r1'!I10, 'r2'!I10, 'r3'!I10, 'r4'!I10)</f>
         <v>0</v>
       </c>
     </row>
@@ -3857,35 +4577,35 @@
         <v>51</v>
       </c>
       <c r="B11">
-        <f>AVERAGE(r0!B11,'r1'!B11, 'r2'!B11, 'r3'!B11)</f>
+        <f>AVERAGE(r0!B11,'r1'!B11, 'r2'!B11, 'r3'!B11, 'r4'!B11)</f>
         <v>0</v>
       </c>
       <c r="C11" s="1">
-        <f>AVERAGE(r0!C11,'r1'!C11, 'r2'!C11, 'r3'!C11)</f>
-        <v>0.5</v>
+        <f>AVERAGE(r0!C11,'r1'!C11, 'r2'!C11, 'r3'!C11, 'r4'!C11)</f>
+        <v>0.6</v>
       </c>
       <c r="D11">
-        <f>AVERAGE(r0!D11,'r1'!D11, 'r2'!D11, 'r3'!D11)</f>
+        <f>AVERAGE(r0!D11,'r1'!D11, 'r2'!D11, 'r3'!D11, 'r4'!D11)</f>
         <v>0</v>
       </c>
       <c r="E11">
-        <f>AVERAGE(r0!E11,'r1'!E11, 'r2'!E11, 'r3'!E11)</f>
+        <f>AVERAGE(r0!E11,'r1'!E11, 'r2'!E11, 'r3'!E11, 'r4'!E11)</f>
         <v>0</v>
       </c>
       <c r="F11">
-        <f>AVERAGE(r0!F11,'r1'!F11, 'r2'!F11, 'r3'!F11)</f>
+        <f>AVERAGE(r0!F11,'r1'!F11, 'r2'!F11, 'r3'!F11, 'r4'!F11)</f>
         <v>0</v>
       </c>
       <c r="G11">
-        <f>AVERAGE(r0!G11,'r1'!G11, 'r2'!G11, 'r3'!G11)</f>
+        <f>AVERAGE(r0!G11,'r1'!G11, 'r2'!G11, 'r3'!G11, 'r4'!G11)</f>
         <v>0</v>
       </c>
       <c r="H11">
-        <f>AVERAGE(r0!H11,'r1'!H11, 'r2'!H11, 'r3'!H11)</f>
+        <f>AVERAGE(r0!H11,'r1'!H11, 'r2'!H11, 'r3'!H11, 'r4'!H11)</f>
         <v>0</v>
       </c>
       <c r="I11">
-        <f>AVERAGE(r0!I11,'r1'!I11, 'r2'!I11, 'r3'!I11)</f>
+        <f>AVERAGE(r0!I11,'r1'!I11, 'r2'!I11, 'r3'!I11, 'r4'!I11)</f>
         <v>0</v>
       </c>
     </row>
@@ -3894,35 +4614,35 @@
         <v>52</v>
       </c>
       <c r="B12">
-        <f>AVERAGE(r0!B12,'r1'!B12, 'r2'!B12, 'r3'!B12)</f>
+        <f>AVERAGE(r0!B12,'r1'!B12, 'r2'!B12, 'r3'!B12, 'r4'!B12)</f>
         <v>0</v>
       </c>
       <c r="C12">
-        <f>AVERAGE(r0!C12,'r1'!C12, 'r2'!C12, 'r3'!C12)</f>
+        <f>AVERAGE(r0!C12,'r1'!C12, 'r2'!C12, 'r3'!C12, 'r4'!C12)</f>
         <v>0</v>
       </c>
       <c r="D12">
-        <f>AVERAGE(r0!D12,'r1'!D12, 'r2'!D12, 'r3'!D12)</f>
+        <f>AVERAGE(r0!D12,'r1'!D12, 'r2'!D12, 'r3'!D12, 'r4'!D12)</f>
         <v>0</v>
       </c>
       <c r="E12">
-        <f>AVERAGE(r0!E12,'r1'!E12, 'r2'!E12, 'r3'!E12)</f>
+        <f>AVERAGE(r0!E12,'r1'!E12, 'r2'!E12, 'r3'!E12, 'r4'!E12)</f>
         <v>0</v>
       </c>
       <c r="F12">
-        <f>AVERAGE(r0!F12,'r1'!F12, 'r2'!F12, 'r3'!F12)</f>
+        <f>AVERAGE(r0!F12,'r1'!F12, 'r2'!F12, 'r3'!F12, 'r4'!F12)</f>
         <v>0</v>
       </c>
       <c r="G12">
-        <f>AVERAGE(r0!G12,'r1'!G12, 'r2'!G12, 'r3'!G12)</f>
+        <f>AVERAGE(r0!G12,'r1'!G12, 'r2'!G12, 'r3'!G12, 'r4'!G12)</f>
         <v>0</v>
       </c>
       <c r="H12">
-        <f>AVERAGE(r0!H12,'r1'!H12, 'r2'!H12, 'r3'!H12)</f>
+        <f>AVERAGE(r0!H12,'r1'!H12, 'r2'!H12, 'r3'!H12, 'r4'!H12)</f>
         <v>0</v>
       </c>
       <c r="I12">
-        <f>AVERAGE(r0!I12,'r1'!I12, 'r2'!I12, 'r3'!I12)</f>
+        <f>AVERAGE(r0!I12,'r1'!I12, 'r2'!I12, 'r3'!I12, 'r4'!I12)</f>
         <v>0</v>
       </c>
     </row>
@@ -3931,35 +4651,35 @@
         <v>53</v>
       </c>
       <c r="B13">
-        <f>AVERAGE(r0!B13,'r1'!B13, 'r2'!B13, 'r3'!B13)</f>
+        <f>AVERAGE(r0!B13,'r1'!B13, 'r2'!B13, 'r3'!B13, 'r4'!B13)</f>
         <v>0</v>
       </c>
       <c r="C13" s="1">
-        <f>AVERAGE(r0!C13,'r1'!C13, 'r2'!C13, 'r3'!C13)</f>
-        <v>0.5</v>
+        <f>AVERAGE(r0!C13,'r1'!C13, 'r2'!C13, 'r3'!C13, 'r4'!C13)</f>
+        <v>0.4</v>
       </c>
       <c r="D13">
-        <f>AVERAGE(r0!D13,'r1'!D13, 'r2'!D13, 'r3'!D13)</f>
+        <f>AVERAGE(r0!D13,'r1'!D13, 'r2'!D13, 'r3'!D13, 'r4'!D13)</f>
         <v>0</v>
       </c>
       <c r="E13">
-        <f>AVERAGE(r0!E13,'r1'!E13, 'r2'!E13, 'r3'!E13)</f>
+        <f>AVERAGE(r0!E13,'r1'!E13, 'r2'!E13, 'r3'!E13, 'r4'!E13)</f>
         <v>0</v>
       </c>
       <c r="F13">
-        <f>AVERAGE(r0!F13,'r1'!F13, 'r2'!F13, 'r3'!F13)</f>
+        <f>AVERAGE(r0!F13,'r1'!F13, 'r2'!F13, 'r3'!F13, 'r4'!F13)</f>
         <v>0</v>
       </c>
       <c r="G13">
-        <f>AVERAGE(r0!G13,'r1'!G13, 'r2'!G13, 'r3'!G13)</f>
+        <f>AVERAGE(r0!G13,'r1'!G13, 'r2'!G13, 'r3'!G13, 'r4'!G13)</f>
         <v>0</v>
       </c>
       <c r="H13">
-        <f>AVERAGE(r0!H13,'r1'!H13, 'r2'!H13, 'r3'!H13)</f>
+        <f>AVERAGE(r0!H13,'r1'!H13, 'r2'!H13, 'r3'!H13, 'r4'!H13)</f>
         <v>0</v>
       </c>
       <c r="I13">
-        <f>AVERAGE(r0!I13,'r1'!I13, 'r2'!I13, 'r3'!I13)</f>
+        <f>AVERAGE(r0!I13,'r1'!I13, 'r2'!I13, 'r3'!I13, 'r4'!I13)</f>
         <v>0</v>
       </c>
     </row>
@@ -3968,35 +4688,35 @@
         <v>9</v>
       </c>
       <c r="B14">
-        <f>AVERAGE(r0!B14,'r1'!B14, 'r2'!B14, 'r3'!B14)</f>
+        <f>AVERAGE(r0!B14,'r1'!B14, 'r2'!B14, 'r3'!B14, 'r4'!B14)</f>
         <v>3</v>
       </c>
       <c r="C14">
-        <f>AVERAGE(r0!C14,'r1'!C14, 'r2'!C14, 'r3'!C14)</f>
+        <f>AVERAGE(r0!C14,'r1'!C14, 'r2'!C14, 'r3'!C14, 'r4'!C14)</f>
         <v>1</v>
       </c>
       <c r="D14">
-        <f>AVERAGE(r0!D14,'r1'!D14, 'r2'!D14, 'r3'!D14)</f>
+        <f>AVERAGE(r0!D14,'r1'!D14, 'r2'!D14, 'r3'!D14, 'r4'!D14)</f>
         <v>1</v>
       </c>
       <c r="E14">
-        <f>AVERAGE(r0!E14,'r1'!E14, 'r2'!E14, 'r3'!E14)</f>
+        <f>AVERAGE(r0!E14,'r1'!E14, 'r2'!E14, 'r3'!E14, 'r4'!E14)</f>
         <v>1</v>
       </c>
       <c r="F14">
-        <f>AVERAGE(r0!F14,'r1'!F14, 'r2'!F14, 'r3'!F14)</f>
+        <f>AVERAGE(r0!F14,'r1'!F14, 'r2'!F14, 'r3'!F14, 'r4'!F14)</f>
         <v>1</v>
       </c>
       <c r="G14">
-        <f>AVERAGE(r0!G14,'r1'!G14, 'r2'!G14, 'r3'!G14)</f>
+        <f>AVERAGE(r0!G14,'r1'!G14, 'r2'!G14, 'r3'!G14, 'r4'!G14)</f>
         <v>1</v>
       </c>
       <c r="H14">
-        <f>AVERAGE(r0!H14,'r1'!H14, 'r2'!H14, 'r3'!H14)</f>
+        <f>AVERAGE(r0!H14,'r1'!H14, 'r2'!H14, 'r3'!H14, 'r4'!H14)</f>
         <v>1</v>
       </c>
       <c r="I14">
-        <f>AVERAGE(r0!I14,'r1'!I14, 'r2'!I14, 'r3'!I14)</f>
+        <f>AVERAGE(r0!I14,'r1'!I14, 'r2'!I14, 'r3'!I14, 'r4'!I14)</f>
         <v>2</v>
       </c>
     </row>
@@ -4005,35 +4725,35 @@
         <v>10</v>
       </c>
       <c r="B15">
-        <f>AVERAGE(r0!B15,'r1'!B15, 'r2'!B15, 'r3'!B15)</f>
+        <f>AVERAGE(r0!B15,'r1'!B15, 'r2'!B15, 'r3'!B15, 'r4'!B15)</f>
         <v>0</v>
       </c>
       <c r="C15">
-        <f>AVERAGE(r0!C15,'r1'!C15, 'r2'!C15, 'r3'!C15)</f>
+        <f>AVERAGE(r0!C15,'r1'!C15, 'r2'!C15, 'r3'!C15, 'r4'!C15)</f>
         <v>0</v>
       </c>
       <c r="D15">
-        <f>AVERAGE(r0!D15,'r1'!D15, 'r2'!D15, 'r3'!D15)</f>
+        <f>AVERAGE(r0!D15,'r1'!D15, 'r2'!D15, 'r3'!D15, 'r4'!D15)</f>
         <v>0</v>
       </c>
       <c r="E15">
-        <f>AVERAGE(r0!E15,'r1'!E15, 'r2'!E15, 'r3'!E15)</f>
+        <f>AVERAGE(r0!E15,'r1'!E15, 'r2'!E15, 'r3'!E15, 'r4'!E15)</f>
         <v>0</v>
       </c>
       <c r="F15">
-        <f>AVERAGE(r0!F15,'r1'!F15, 'r2'!F15, 'r3'!F15)</f>
+        <f>AVERAGE(r0!F15,'r1'!F15, 'r2'!F15, 'r3'!F15, 'r4'!F15)</f>
         <v>1</v>
       </c>
       <c r="G15">
-        <f>AVERAGE(r0!G15,'r1'!G15, 'r2'!G15, 'r3'!G15)</f>
+        <f>AVERAGE(r0!G15,'r1'!G15, 'r2'!G15, 'r3'!G15, 'r4'!G15)</f>
         <v>0</v>
       </c>
       <c r="H15">
-        <f>AVERAGE(r0!H15,'r1'!H15, 'r2'!H15, 'r3'!H15)</f>
+        <f>AVERAGE(r0!H15,'r1'!H15, 'r2'!H15, 'r3'!H15, 'r4'!H15)</f>
         <v>1</v>
       </c>
       <c r="I15">
-        <f>AVERAGE(r0!I15,'r1'!I15, 'r2'!I15, 'r3'!I15)</f>
+        <f>AVERAGE(r0!I15,'r1'!I15, 'r2'!I15, 'r3'!I15, 'r4'!I15)</f>
         <v>0</v>
       </c>
     </row>
@@ -4042,36 +4762,36 @@
         <v>11</v>
       </c>
       <c r="B16">
-        <f>AVERAGE(r0!B16,'r1'!B16, 'r2'!B16, 'r3'!B16)</f>
+        <f>AVERAGE(r0!B16,'r1'!B16, 'r2'!B16, 'r3'!B16, 'r4'!B16)</f>
         <v>3</v>
       </c>
       <c r="C16">
-        <f>AVERAGE(r0!C16,'r1'!C16, 'r2'!C16, 'r3'!C16)</f>
+        <f>AVERAGE(r0!C16,'r1'!C16, 'r2'!C16, 'r3'!C16, 'r4'!C16)</f>
         <v>1</v>
       </c>
       <c r="D16">
-        <f>AVERAGE(r0!D16,'r1'!D16, 'r2'!D16, 'r3'!D16)</f>
+        <f>AVERAGE(r0!D16,'r1'!D16, 'r2'!D16, 'r3'!D16, 'r4'!D16)</f>
         <v>1</v>
       </c>
       <c r="E16">
-        <f>AVERAGE(r0!E16,'r1'!E16, 'r2'!E16, 'r3'!E16)</f>
+        <f>AVERAGE(r0!E16,'r1'!E16, 'r2'!E16, 'r3'!E16, 'r4'!E16)</f>
         <v>1</v>
       </c>
       <c r="F16">
-        <f>AVERAGE(r0!F16,'r1'!F16, 'r2'!F16, 'r3'!F16)</f>
+        <f>AVERAGE(r0!F16,'r1'!F16, 'r2'!F16, 'r3'!F16, 'r4'!F16)</f>
         <v>1</v>
       </c>
       <c r="G16">
-        <f>AVERAGE(r0!G16,'r1'!G16, 'r2'!G16, 'r3'!G16)</f>
+        <f>AVERAGE(r0!G16,'r1'!G16, 'r2'!G16, 'r3'!G16, 'r4'!G16)</f>
         <v>1</v>
       </c>
       <c r="H16">
-        <f>AVERAGE(r0!H16,'r1'!H16, 'r2'!H16, 'r3'!H16)</f>
-        <v>1</v>
-      </c>
-      <c r="I16" s="1">
-        <f>AVERAGE(r0!I16,'r1'!I16, 'r2'!I16, 'r3'!I16)</f>
-        <v>1.75</v>
+        <f>AVERAGE(r0!H16,'r1'!H16, 'r2'!H16, 'r3'!H16, 'r4'!H16)</f>
+        <v>1</v>
+      </c>
+      <c r="I16" s="5">
+        <f>AVERAGE(r0!I16,'r1'!I16, 'r2'!I16, 'r3'!I16, 'r4'!I16)</f>
+        <v>2</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
@@ -4079,36 +4799,36 @@
         <v>12</v>
       </c>
       <c r="B17">
-        <f>AVERAGE(r0!B17,'r1'!B17, 'r2'!B17, 'r3'!B17)</f>
+        <f>AVERAGE(r0!B17,'r1'!B17, 'r2'!B17, 'r3'!B17, 'r4'!B17)</f>
         <v>3</v>
       </c>
       <c r="C17">
-        <f>AVERAGE(r0!C17,'r1'!C17, 'r2'!C17, 'r3'!C17)</f>
+        <f>AVERAGE(r0!C17,'r1'!C17, 'r2'!C17, 'r3'!C17, 'r4'!C17)</f>
         <v>1</v>
       </c>
       <c r="D17">
-        <f>AVERAGE(r0!D17,'r1'!D17, 'r2'!D17, 'r3'!D17)</f>
+        <f>AVERAGE(r0!D17,'r1'!D17, 'r2'!D17, 'r3'!D17, 'r4'!D17)</f>
         <v>1</v>
       </c>
       <c r="E17">
-        <f>AVERAGE(r0!E17,'r1'!E17, 'r2'!E17, 'r3'!E17)</f>
+        <f>AVERAGE(r0!E17,'r1'!E17, 'r2'!E17, 'r3'!E17, 'r4'!E17)</f>
         <v>1</v>
       </c>
       <c r="F17">
-        <f>AVERAGE(r0!F17,'r1'!F17, 'r2'!F17, 'r3'!F17)</f>
+        <f>AVERAGE(r0!F17,'r1'!F17, 'r2'!F17, 'r3'!F17, 'r4'!F17)</f>
         <v>1</v>
       </c>
       <c r="G17">
-        <f>AVERAGE(r0!G17,'r1'!G17, 'r2'!G17, 'r3'!G17)</f>
+        <f>AVERAGE(r0!G17,'r1'!G17, 'r2'!G17, 'r3'!G17, 'r4'!G17)</f>
         <v>1</v>
       </c>
       <c r="H17">
-        <f>AVERAGE(r0!H17,'r1'!H17, 'r2'!H17, 'r3'!H17)</f>
-        <v>1</v>
-      </c>
-      <c r="I17" s="1">
-        <f>AVERAGE(r0!I17,'r1'!I17, 'r2'!I17, 'r3'!I17)</f>
-        <v>1.75</v>
+        <f>AVERAGE(r0!H17,'r1'!H17, 'r2'!H17, 'r3'!H17, 'r4'!H17)</f>
+        <v>1</v>
+      </c>
+      <c r="I17" s="5">
+        <f>AVERAGE(r0!I17,'r1'!I17, 'r2'!I17, 'r3'!I17, 'r4'!I17)</f>
+        <v>2</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
@@ -4116,35 +4836,35 @@
         <v>13</v>
       </c>
       <c r="B18" s="1">
-        <f>AVERAGE(r0!B18,'r1'!B18, 'r2'!B18, 'r3'!B18)</f>
-        <v>0.75</v>
+        <f>AVERAGE(r0!B18,'r1'!B18, 'r2'!B18, 'r3'!B18, 'r4'!B18)</f>
+        <v>0.6</v>
       </c>
       <c r="C18" s="1">
-        <f>AVERAGE(r0!C18,'r1'!C18, 'r2'!C18, 'r3'!C18)</f>
-        <v>0.5</v>
+        <f>AVERAGE(r0!C18,'r1'!C18, 'r2'!C18, 'r3'!C18, 'r4'!C18)</f>
+        <v>0.4</v>
       </c>
       <c r="D18">
-        <f>AVERAGE(r0!D18,'r1'!D18, 'r2'!D18, 'r3'!D18)</f>
+        <f>AVERAGE(r0!D18,'r1'!D18, 'r2'!D18, 'r3'!D18, 'r4'!D18)</f>
         <v>0</v>
       </c>
       <c r="E18">
-        <f>AVERAGE(r0!E18,'r1'!E18, 'r2'!E18, 'r3'!E18)</f>
+        <f>AVERAGE(r0!E18,'r1'!E18, 'r2'!E18, 'r3'!E18, 'r4'!E18)</f>
         <v>0</v>
       </c>
       <c r="F18">
-        <f>AVERAGE(r0!F18,'r1'!F18, 'r2'!F18, 'r3'!F18)</f>
+        <f>AVERAGE(r0!F18,'r1'!F18, 'r2'!F18, 'r3'!F18, 'r4'!F18)</f>
         <v>0</v>
       </c>
       <c r="G18">
-        <f>AVERAGE(r0!G18,'r1'!G18, 'r2'!G18, 'r3'!G18)</f>
+        <f>AVERAGE(r0!G18,'r1'!G18, 'r2'!G18, 'r3'!G18, 'r4'!G18)</f>
         <v>0</v>
       </c>
       <c r="H18">
-        <f>AVERAGE(r0!H18,'r1'!H18, 'r2'!H18, 'r3'!H18)</f>
+        <f>AVERAGE(r0!H18,'r1'!H18, 'r2'!H18, 'r3'!H18, 'r4'!H18)</f>
         <v>0</v>
       </c>
       <c r="I18">
-        <f>AVERAGE(r0!I18,'r1'!I18, 'r2'!I18, 'r3'!I18)</f>
+        <f>AVERAGE(r0!I18,'r1'!I18, 'r2'!I18, 'r3'!I18, 'r4'!I18)</f>
         <v>0</v>
       </c>
     </row>
@@ -4153,35 +4873,35 @@
         <v>14</v>
       </c>
       <c r="B19">
-        <f>AVERAGE(r0!B19,'r1'!B19, 'r2'!B19, 'r3'!B19)</f>
+        <f>AVERAGE(r0!B19,'r1'!B19, 'r2'!B19, 'r3'!B19, 'r4'!B19)</f>
         <v>0</v>
       </c>
       <c r="C19">
-        <f>AVERAGE(r0!C19,'r1'!C19, 'r2'!C19, 'r3'!C19)</f>
+        <f>AVERAGE(r0!C19,'r1'!C19, 'r2'!C19, 'r3'!C19, 'r4'!C19)</f>
         <v>0</v>
       </c>
       <c r="D19">
-        <f>AVERAGE(r0!D19,'r1'!D19, 'r2'!D19, 'r3'!D19)</f>
+        <f>AVERAGE(r0!D19,'r1'!D19, 'r2'!D19, 'r3'!D19, 'r4'!D19)</f>
         <v>0</v>
       </c>
       <c r="E19">
-        <f>AVERAGE(r0!E19,'r1'!E19, 'r2'!E19, 'r3'!E19)</f>
+        <f>AVERAGE(r0!E19,'r1'!E19, 'r2'!E19, 'r3'!E19, 'r4'!E19)</f>
         <v>0</v>
       </c>
       <c r="F19">
-        <f>AVERAGE(r0!F19,'r1'!F19, 'r2'!F19, 'r3'!F19)</f>
+        <f>AVERAGE(r0!F19,'r1'!F19, 'r2'!F19, 'r3'!F19, 'r4'!F19)</f>
         <v>0</v>
       </c>
       <c r="G19">
-        <f>AVERAGE(r0!G19,'r1'!G19, 'r2'!G19, 'r3'!G19)</f>
+        <f>AVERAGE(r0!G19,'r1'!G19, 'r2'!G19, 'r3'!G19, 'r4'!G19)</f>
         <v>0</v>
       </c>
       <c r="H19">
-        <f>AVERAGE(r0!H19,'r1'!H19, 'r2'!H19, 'r3'!H19)</f>
+        <f>AVERAGE(r0!H19,'r1'!H19, 'r2'!H19, 'r3'!H19, 'r4'!H19)</f>
         <v>0</v>
       </c>
       <c r="I19">
-        <f>AVERAGE(r0!I19,'r1'!I19, 'r2'!I19, 'r3'!I19)</f>
+        <f>AVERAGE(r0!I19,'r1'!I19, 'r2'!I19, 'r3'!I19, 'r4'!I19)</f>
         <v>0</v>
       </c>
     </row>
@@ -4190,35 +4910,35 @@
         <v>15</v>
       </c>
       <c r="B20">
-        <f>AVERAGE(r0!B20,'r1'!B20, 'r2'!B20, 'r3'!B20)</f>
+        <f>AVERAGE(r0!B20,'r1'!B20, 'r2'!B20, 'r3'!B20, 'r4'!B20)</f>
         <v>0</v>
       </c>
       <c r="C20">
-        <f>AVERAGE(r0!C20,'r1'!C20, 'r2'!C20, 'r3'!C20)</f>
-        <v>0</v>
-      </c>
-      <c r="D20">
-        <f>AVERAGE(r0!D20,'r1'!D20, 'r2'!D20, 'r3'!D20)</f>
-        <v>0.5</v>
+        <f>AVERAGE(r0!C20,'r1'!C20, 'r2'!C20, 'r3'!C20, 'r4'!C20)</f>
+        <v>0</v>
+      </c>
+      <c r="D20" s="1">
+        <f>AVERAGE(r0!D20,'r1'!D20, 'r2'!D20, 'r3'!D20, 'r4'!D20)</f>
+        <v>0.4</v>
       </c>
       <c r="E20">
-        <f>AVERAGE(r0!E20,'r1'!E20, 'r2'!E20, 'r3'!E20)</f>
+        <f>AVERAGE(r0!E20,'r1'!E20, 'r2'!E20, 'r3'!E20, 'r4'!E20)</f>
         <v>0</v>
       </c>
       <c r="F20" s="1">
-        <f>AVERAGE(r0!F20,'r1'!F20, 'r2'!F20, 'r3'!F20)</f>
-        <v>0.75</v>
+        <f>AVERAGE(r0!F20,'r1'!F20, 'r2'!F20, 'r3'!F20, 'r4'!F20)</f>
+        <v>0.8</v>
       </c>
       <c r="G20">
-        <f>AVERAGE(r0!G20,'r1'!G20, 'r2'!G20, 'r3'!G20)</f>
-        <v>1</v>
+        <f>AVERAGE(r0!G20,'r1'!G20, 'r2'!G20, 'r3'!G20, 'r4'!G20)</f>
+        <v>0.8</v>
       </c>
       <c r="H20">
-        <f>AVERAGE(r0!H20,'r1'!H20, 'r2'!H20, 'r3'!H20)</f>
+        <f>AVERAGE(r0!H20,'r1'!H20, 'r2'!H20, 'r3'!H20, 'r4'!H20)</f>
         <v>0</v>
       </c>
       <c r="I20">
-        <f>AVERAGE(r0!I20,'r1'!I20, 'r2'!I20, 'r3'!I20)</f>
+        <f>AVERAGE(r0!I20,'r1'!I20, 'r2'!I20, 'r3'!I20, 'r4'!I20)</f>
         <v>1</v>
       </c>
     </row>
@@ -4227,36 +4947,36 @@
         <v>55</v>
       </c>
       <c r="B21" s="1">
-        <f>AVERAGE(r0!B21,'r1'!B21, 'r2'!B21, 'r3'!B21)</f>
-        <v>25.304000000000002</v>
+        <f>AVERAGE(r0!B21,'r1'!B21, 'r2'!B21, 'r3'!B21, 'r4'!B21)</f>
+        <v>24.785400000000003</v>
       </c>
       <c r="C21" s="1">
-        <f>AVERAGE(r0!C21,'r1'!C21, 'r2'!C21, 'r3'!C21)</f>
-        <v>21.376249999999999</v>
+        <f>AVERAGE(r0!C21,'r1'!C21, 'r2'!C21, 'r3'!C21, 'r4'!C21)</f>
+        <v>20.919999999999998</v>
       </c>
       <c r="D21" s="1">
-        <f>AVERAGE(r0!D21,'r1'!D21, 'r2'!D21, 'r3'!D21)</f>
-        <v>15.272</v>
+        <f>AVERAGE(r0!D21,'r1'!D21, 'r2'!D21, 'r3'!D21, 'r4'!D21)</f>
+        <v>14.699199999999999</v>
       </c>
       <c r="E21" s="1">
-        <f>AVERAGE(r0!E21,'r1'!E21, 'r2'!E21, 'r3'!E21)</f>
-        <v>17.91075</v>
+        <f>AVERAGE(r0!E21,'r1'!E21, 'r2'!E21, 'r3'!E21, 'r4'!E21)</f>
+        <v>17.506399999999999</v>
       </c>
       <c r="F21" s="1">
-        <f>AVERAGE(r0!F21,'r1'!F21, 'r2'!F21, 'r3'!F21)</f>
-        <v>13.00375</v>
+        <f>AVERAGE(r0!F21,'r1'!F21, 'r2'!F21, 'r3'!F21, 'r4'!F21)</f>
+        <v>13.018799999999999</v>
       </c>
       <c r="G21" s="1">
-        <f>AVERAGE(r0!G21,'r1'!G21, 'r2'!G21, 'r3'!G21)</f>
-        <v>12.51925</v>
+        <f>AVERAGE(r0!G21,'r1'!G21, 'r2'!G21, 'r3'!G21, 'r4'!G21)</f>
+        <v>11.556999999999999</v>
       </c>
       <c r="H21" s="1">
-        <f>AVERAGE(r0!H21,'r1'!H21, 'r2'!H21, 'r3'!H21)</f>
-        <v>16.987500000000001</v>
+        <f>AVERAGE(r0!H21,'r1'!H21, 'r2'!H21, 'r3'!H21, 'r4'!H21)</f>
+        <v>15.855</v>
       </c>
       <c r="I21" s="1">
-        <f>AVERAGE(r0!I21,'r1'!I21, 'r2'!I21, 'r3'!I21)</f>
-        <v>15.70975</v>
+        <f>AVERAGE(r0!I21,'r1'!I21, 'r2'!I21, 'r3'!I21, 'r4'!I21)</f>
+        <v>15.277799999999999</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -4264,53 +4984,73 @@
         <v>54</v>
       </c>
       <c r="B22" s="1">
-        <f>AVERAGE(r0!B22,'r1'!B22, 'r2'!B22, 'r3'!B22)</f>
-        <v>2.4203500000000003E-2</v>
+        <f>AVERAGE(r0!B22,'r1'!B22, 'r2'!B22, 'r3'!B22, 'r4'!B22)</f>
+        <v>2.4224200000000001E-2</v>
       </c>
       <c r="C22" s="1">
-        <f>AVERAGE(r0!C22,'r1'!C22, 'r2'!C22, 'r3'!C22)</f>
-        <v>2.2918250000000001E-2</v>
+        <f>AVERAGE(r0!C22,'r1'!C22, 'r2'!C22, 'r3'!C22, 'r4'!C22)</f>
+        <v>2.2412400000000002E-2</v>
       </c>
       <c r="D22" s="1">
-        <f>AVERAGE(r0!D22,'r1'!D22, 'r2'!D22, 'r3'!D22)</f>
-        <v>1.7138500000000001E-2</v>
+        <f>AVERAGE(r0!D22,'r1'!D22, 'r2'!D22, 'r3'!D22, 'r4'!D22)</f>
+        <v>1.6243E-2</v>
       </c>
       <c r="E22" s="1">
-        <f>AVERAGE(r0!E22,'r1'!E22, 'r2'!E22, 'r3'!E22)</f>
-        <v>1.9991000000000002E-2</v>
+        <f>AVERAGE(r0!E22,'r1'!E22, 'r2'!E22, 'r3'!E22, 'r4'!E22)</f>
+        <v>1.9662200000000001E-2</v>
       </c>
       <c r="F22" s="1">
-        <f>AVERAGE(r0!F22,'r1'!F22, 'r2'!F22, 'r3'!F22)</f>
-        <v>1.516175E-2</v>
+        <f>AVERAGE(r0!F22,'r1'!F22, 'r2'!F22, 'r3'!F22, 'r4'!F22)</f>
+        <v>1.47972E-2</v>
       </c>
       <c r="G22" s="1">
-        <f>AVERAGE(r0!G22,'r1'!G22, 'r2'!G22, 'r3'!G22)</f>
-        <v>1.2981999999999999E-2</v>
+        <f>AVERAGE(r0!G22,'r1'!G22, 'r2'!G22, 'r3'!G22, 'r4'!G22)</f>
+        <v>1.2199199999999999E-2</v>
       </c>
       <c r="H22" s="1">
-        <f>AVERAGE(r0!H22,'r1'!H22, 'r2'!H22, 'r3'!H22)</f>
-        <v>1.50215E-2</v>
+        <f>AVERAGE(r0!H22,'r1'!H22, 'r2'!H22, 'r3'!H22, 'r4'!H22)</f>
+        <v>1.4433000000000001E-2</v>
       </c>
       <c r="I22" s="1">
-        <f>AVERAGE(r0!I22,'r1'!I22, 'r2'!I22, 'r3'!I22)</f>
-        <v>1.7203E-2</v>
+        <f>AVERAGE(r0!I22,'r1'!I22, 'r2'!I22, 'r3'!I22, 'r4'!I22)</f>
+        <v>1.6671399999999999E-2</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
-      <c r="F23" s="2"/>
-      <c r="G23" s="2"/>
-      <c r="H23" s="2"/>
-      <c r="I23" s="2"/>
+      <c r="A23" t="s">
+        <v>17</v>
+      </c>
+      <c r="B23" t="s">
+        <v>18</v>
+      </c>
+      <c r="C23" t="s">
+        <v>18</v>
+      </c>
+      <c r="D23" t="s">
+        <v>18</v>
+      </c>
+      <c r="E23" t="s">
+        <v>18</v>
+      </c>
+      <c r="F23" t="s">
+        <v>18</v>
+      </c>
+      <c r="G23" t="s">
+        <v>18</v>
+      </c>
+      <c r="H23" t="s">
+        <v>18</v>
+      </c>
+      <c r="I23" t="s">
+        <v>18</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE3232CA-EC8E-404A-B90B-03381B7790AE}">
   <dimension ref="A1:I23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>